<commit_message>
auto sync 2026-06-12 05:50:01
</commit_message>
<xml_diff>
--- a/Marathon_programme.xlsx
+++ b/Marathon_programme.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Préparation IM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation IM Final V2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,11 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,15 +41,24 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -64,7 +72,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0037474F"/>
+        <fgColor rgb="00795548"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,12 +92,52 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFCCBC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E65100"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00880E4F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A148C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0037474F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000277BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B71C1C"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,7 +175,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -148,13 +196,43 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -536,6 +614,7 @@
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -594,15 +673,20 @@
           <t>Distance (m) - Natation</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>D+</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Semaine 1 — 01/06 au 07/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="39" customHeight="1">
+          <t xml:space="preserve">  03/06 → 07/06/2026   |   Récupération totale — Pas de vélo, pas de CAP | Nat WE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="52" customHeight="1">
       <c r="A3" s="3" t="n">
         <v>46176</v>
       </c>
@@ -636,14 +720,16 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>J+18 marathon — Repos complet
+          <t>J+18 marathon — Repos COMPLET
 Pas de course, pas de vélo
-Le corps est encore en récupération profonde</t>
+Le corps est encore en récupération profonde
+Genou : observer l'évolution de la douleur face avant</t>
         </is>
       </c>
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -686,6 +772,7 @@
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -727,6 +814,7 @@
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -771,6 +859,7 @@
       <c r="K6" s="4" t="n">
         <v>1000</v>
       </c>
+      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7" ht="39" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -814,6 +903,7 @@
       <c r="K7" s="4" t="n">
         <v>1000</v>
       </c>
+      <c r="L7" s="4" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="9" t="n"/>
@@ -825,7 +915,7 @@
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I8" s="9" t="n"/>
@@ -833,11 +923,12 @@
       <c r="K8" s="9" t="n">
         <v>2000</v>
       </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 2 — 08/06 au 14/06/2026</t>
+      <c r="L8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  08/06 → 14/06/2026   |   Retour CAP très progressif PLAT STRICT — Pas de vélo | Nat WE</t>
         </is>
       </c>
     </row>
@@ -881,8 +972,9 @@
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="65" customHeight="1">
+      <c r="L10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="104" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>46182</v>
       </c>
@@ -891,14 +983,14 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Test reprise CAP — EF très court</t>
+          <t>Test reprise CAP — Marche-course PLAT STRICT</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
@@ -915,10 +1007,13 @@
       <c r="H11" s="7" t="inlineStr">
         <is>
           <t>PREMIER TEST REPRISE CAP — J+24 marathon
-18' de marche-course Z1 (&lt;128 bpm)
-Si douleur : s'arrêter immédiatement et revenir à du repos
-Si OK : noter les sensations pour adapter la suite
-Allure très lente — marche si besoin</t>
+PROTOCOLE GENOU :
+  · TERRAIN PLAT UNIQUEMENT — zéro côte, zéro escalier, zéro trottoir en pente
+  · Marche-course : 1 min course / 1 min marche — alterner
+  · FC &lt; 128 bpm — allure très lente
+  · Si douleur &gt; 3/10 : ARRÊT IMMÉDIAT — retour repos complet
+  · Si OK : noter la douleur /10 avant, pendant, après
+PAS de trail, PAS de pente, PAS de dénivelé</t>
         </is>
       </c>
       <c r="I11" s="4" t="n">
@@ -926,8 +1021,11 @@
       </c>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="26" customHeight="1">
+      <c r="L11" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" ht="39" customHeight="1">
       <c r="A12" s="3" t="n">
         <v>46183</v>
       </c>
@@ -962,14 +1060,16 @@
       <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Repos — observer les sensations post-test
-Si douleurs : allonger la période de repos</t>
+Si douleurs : allonger la période de repos
+Genou : noter douleur au repos, à la montée des escaliers</t>
         </is>
       </c>
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="52" customHeight="1">
+      <c r="L12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="91" customHeight="1">
       <c r="A13" s="3" t="n">
         <v>46184</v>
       </c>
@@ -978,14 +1078,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>EF très léger — si sensations OK</t>
+          <t>EF très léger — PLAT STRICT (si test mardi OK)</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
@@ -1002,9 +1102,12 @@
       <c r="H13" s="7" t="inlineStr">
         <is>
           <t>22' marche-course (120-130 bpm)
-SEULEMENT si le test mardi s'est bien passé
-Sinon : repos complet
-Écouter le corps — aucune pression</t>
+SEULEMENT si mardi s'est passé sans douleur &gt; 2/10
+Sinon : repos complet sans exception
+PROTOCOLE GENOU :
+  · Terrain plat strict — zéro dénivelé
+  · Marche-course si besoin
+  · Surveiller douleur tendon rotulien/quadricipital</t>
         </is>
       </c>
       <c r="I13" s="4" t="n">
@@ -1012,6 +1115,9 @@
       </c>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -1053,6 +1159,7 @@
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1095,6 +1202,7 @@
       <c r="K15" s="4" t="n">
         <v>1200</v>
       </c>
+      <c r="L15" s="4" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1137,6 +1245,7 @@
       <c r="K16" s="4" t="n">
         <v>1200</v>
       </c>
+      <c r="L16" s="4" t="n"/>
     </row>
     <row r="17" ht="39" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1147,14 +1256,14 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>EF très léger post-nat — si OK</t>
+          <t>EF très léger post-nat — PLAT STRICT (si OK)</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1171,7 +1280,7 @@
       <c r="H17" s="7" t="inlineStr">
         <is>
           <t>20' EF Z1 (120-130 bpm) — UNIQUEMENT si pas de douleur
-Marche-course — allure très basse
+Terrain plat strict — marche-course
 Si sensations mauvaises : ne pas faire</t>
         </is>
       </c>
@@ -1180,6 +1289,9 @@
       </c>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="9" t="n"/>
@@ -1191,7 +1303,7 @@
       <c r="G18" s="9" t="n"/>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I18" s="9" t="n">
@@ -1201,11 +1313,12 @@
       <c r="K18" s="9" t="n">
         <v>2400</v>
       </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 3 — 15/06 au 21/06/2026</t>
+      <c r="L18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  15/06 → 21/06/2026   |   Reprise CAP douce PLAT — Pas de vélo | Décision Malaga 20/06</t>
         </is>
       </c>
     </row>
@@ -1249,8 +1362,9 @@
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="39" customHeight="1">
+      <c r="L20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="65" customHeight="1">
       <c r="A21" s="3" t="n">
         <v>46189</v>
       </c>
@@ -1259,14 +1373,14 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>EF douce — 28'</t>
+          <t>EF douce — 28' PLAT STRICT</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
@@ -1282,9 +1396,11 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>28' EF Z1-Z2 (120-135 bpm)
-Allure très facile — pas de tempo, pas de côtes
-Si douleur persiste : réduire à 15' ou annuler</t>
+          <t>28' EF Z1-Z2 (120-135 bpm) — TERRAIN PLAT UNIQUEMENT
+PROTOCOLE GENOU :
+  · Zéro côte, zéro escalier, zéro pente
+  · Si douleur &gt; 2/10 : réduire à 15' ou annuler
+  · Si OK : noter la douleur et l'évolution</t>
         </is>
       </c>
       <c r="I21" s="4" t="n">
@@ -1292,6 +1408,9 @@
       </c>
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -1333,8 +1452,9 @@
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="39" customHeight="1">
+      <c r="L22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="52" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>46191</v>
       </c>
@@ -1343,14 +1463,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>EF douce — 32'</t>
+          <t>EF douce — 32' PLAT STRICT</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
@@ -1366,9 +1486,10 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>32' EF Z1-Z2 (120-135 bpm)
+          <t>32' EF Z1-Z2 (120-135 bpm) — TERRAIN PLAT UNIQUEMENT
 Montée progressive par rapport à mardi
-Écouter le corps</t>
+PROTOCOLE GENOU : zéro dénivelé — surveiller douleur
+Si mardi a bien passé → tenir 32' | Si inconfort → 20' max</t>
         </is>
       </c>
       <c r="I23" s="4" t="n">
@@ -1376,6 +1497,9 @@
       </c>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -1417,8 +1541,9 @@
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
-    </row>
-    <row r="25" ht="26" customHeight="1">
+      <c r="L24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="108" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>46193</v>
       </c>
@@ -1453,12 +1578,20 @@
       <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Voyage Luxembourg→Paris puis nuit Paris
-Pas de séance — voyage</t>
+Pas de séance — voyage
+⚠️ DÉCISION MALAGA — À PRENDRE AUJOURD'HUI :
+Scénario A : CAP 30' sans douleur cette semaine
+  → Plan normal — DESCENTES À PIED obligatoires
+Scénario B : CAP possible mais inconfort
+  → 2-3 montées max/jour — descentes à pied — priorité natation
+Scénario C : Douleur encore présente
+  → ZÉRO course à Malaga — natation uniquement 2x/jour</t>
         </is>
       </c>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="3" t="n">
@@ -1501,6 +1634,7 @@
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="9" t="n"/>
@@ -1512,7 +1646,7 @@
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I27" s="9" t="n">
@@ -1520,15 +1654,16 @@
       </c>
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 4 — 22/06 au 28/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="78" customHeight="1">
+      <c r="L27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  22/06 → 28/06/2026   |   🏔️ CAMP MALAGA — Montées CAP (DESCENTES À PIED) + Nat mer</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="104" customHeight="1">
       <c r="A29" s="3" t="n">
         <v>46195</v>
       </c>
@@ -1537,14 +1672,14 @@
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>🏔️ MALAGA J1 — CAP côte : découverte légère</t>
+          <t>🏔️ MALAGA J1 — Montées uniquement (descentes à pied)</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
@@ -1561,10 +1696,12 @@
       <c r="H29" s="7" t="inlineStr">
         <is>
           <t>CAMP MALAGA — Jour 1 : Très progressif
-10' EF | 3x [Montée 200m D+ @ Z2-Z3 (138-155 bpm) — descente récup Z1] | 15' RC
-FOCUS : écouter le corps — première vraie sortie sérieuse depuis le marathon
-Courir tôt le matin (avant 8h) — chaleur Malaga
-Descentes très lentes — protéger les tendons
+10' EF plat | 3x MONTÉE 200m D+ @ Z2-Z3 (138-155 bpm)
+⚠️ RÈGLE ABSOLUE GENOU : DESCENTES À PIED — jamais en courant
+Les descentes = contraction excentrique quadriceps = aggravation tendinopathie
+Marcher les descentes : 3-4 min de marche active
+Courir tôt (avant 8h) — chaleur Malaga
+Si douleur &gt; 3/10 en montée : STOP — passer scénario C
 D+ cumulé : ~600m</t>
         </is>
       </c>
@@ -1573,6 +1710,9 @@
       </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="30" ht="39" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -1606,7 +1746,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Mer Méditerranée — après-midi (chaleur réduite)
+          <t>Mer Méditerranée — après-midi
 500-700m EF en eau libre
 Sighting obligatoire — récupération musculaire</t>
         </is>
@@ -1616,8 +1756,9 @@
       <c r="K30" s="4" t="n">
         <v>600</v>
       </c>
-    </row>
-    <row r="31" ht="65" customHeight="1">
+      <c r="L30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="78" customHeight="1">
       <c r="A31" s="3" t="n">
         <v>46196</v>
       </c>
@@ -1626,14 +1767,14 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>🏔️ MALAGA J2 — CAP côte : progression</t>
+          <t>🏔️ MALAGA J2 — Montées + descentes à pied</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
@@ -1650,9 +1791,10 @@
       <c r="H31" s="7" t="inlineStr">
         <is>
           <t>CAMP MALAGA — Jour 2 : Build progressif
-10' EF | 4x [Montée 200m D+ @ Z3 (147-160 bpm) — r=3' descente] | 12' RC
-Si J1 bien passé → tenir cette intensité
-Si sensations difficiles → réduire à 3 montées
+10' EF plat | 4x MONTÉE 200m D+ @ Z3 (147-160 bpm)
+⚠️ DESCENTES À PIED — toujours — sans exception
+Durée descente : 3-4 min de marche active
+Si J1 bien passé → 4 montées | Sinon → 3 montées
 D+ cumulé : ~800m</t>
         </is>
       </c>
@@ -1661,8 +1803,11 @@
       </c>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="26" customHeight="1">
+      <c r="L31" s="4" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="3" t="n">
         <v>46196</v>
       </c>
@@ -1694,8 +1839,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>700-800m | 200 EF | 4x75 allure (r=15'') | 300 retour
-Sighting + rythme</t>
+          <t>700-800m | 200 EF | 4x75 allure (r=15'') | 300 retour</t>
         </is>
       </c>
       <c r="I32" s="4" t="n"/>
@@ -1703,6 +1847,7 @@
       <c r="K32" s="4" t="n">
         <v>750</v>
       </c>
+      <c r="L32" s="4" t="n"/>
     </row>
     <row r="33" ht="78" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -1713,14 +1858,14 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>🏔️ MALAGA J3 — CAP côte : séance du camp</t>
+          <t>🏔️ MALAGA J3 — Séance principale (descentes à pied)</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -1737,10 +1882,10 @@
       <c r="H33" s="7" t="inlineStr">
         <is>
           <t>CAMP MALAGA — Jour 3 : Séance principale
-10' EF | 5x [Montée 200m D+ @ Z3 (150-162 bpm) — r=3' descente] | 12' RC
-ADAPTÉ : 5 montées max (pas 9 comme prévu initialement)
+10' EF plat | 5x MONTÉE 200m D+ @ Z3 (150-162 bpm)
+⚠️ DESCENTES À PIED — absolument — règle la plus importante du camp
+Courir les descentes = risque de rechute 2-3 semaines
 Partir tôt (6h) — gel à mi-séance — boire AVANT d'avoir soif
-Descentes LENTES — récup active
 D+ cumulé : ~1 000m</t>
         </is>
       </c>
@@ -1749,6 +1894,9 @@
       </c>
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="34" ht="39" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -1782,7 +1930,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>700-900m EF — récupération après la séance principale
+          <t>700-900m EF — récupération après séance principale
 Eau de mer = récup muscles et tendons
 Pas d'intensité</t>
         </is>
@@ -1792,6 +1940,7 @@
       <c r="K34" s="4" t="n">
         <v>800</v>
       </c>
+      <c r="L34" s="4" t="n"/>
     </row>
     <row r="35" ht="39" customHeight="1">
       <c r="A35" s="3" t="n">
@@ -1829,12 +1978,13 @@
         <is>
           <t>🏔️ MALAGA J4 — Repos / Tourisme
 Journée de récupération active — marche, plage
-Pas de séance structurée — le corps a besoin de récupérer</t>
+Pas de séance structurée</t>
         </is>
       </c>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -1877,8 +2027,9 @@
       <c r="K36" s="4" t="n">
         <v>550</v>
       </c>
-    </row>
-    <row r="37" ht="65" customHeight="1">
+      <c r="L36" s="4" t="n"/>
+    </row>
+    <row r="37" ht="78" customHeight="1">
       <c r="A37" s="3" t="n">
         <v>46199</v>
       </c>
@@ -1887,14 +2038,14 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>🏔️ MALAGA J5 — CAP côte : deuxième session</t>
+          <t>🏔️ MALAGA J5 — Montées (descentes à pied)</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -1910,9 +2061,10 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>CAMP MALAGA — Jour 5 : Deuxième session qualitative
-10' EF | 4x [Montée 200m D+ @ Z3 (148-162 bpm) — r=3' descente] | 12' RC
-Tenir l'intensité malgré fatigue cumulée du camp
+          <t>CAMP MALAGA — Jour 5 : Deuxième session
+10' EF plat | 4x MONTÉE 200m D+ @ Z3 (148-162 bpm)
+⚠️ DESCENTES À PIED — règle non négociable
+Fatigue cumulée → surveiller encore plus le genou
 Si sensations difficiles → 3 montées seulement
 D+ cumulé : ~800m</t>
         </is>
@@ -1922,6 +2074,9 @@
       </c>
       <c r="J37" s="4" t="n"/>
       <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="3" t="n">
@@ -1963,8 +2118,9 @@
       <c r="K38" s="4" t="n">
         <v>800</v>
       </c>
-    </row>
-    <row r="39" ht="52" customHeight="1">
+      <c r="L38" s="4" t="n"/>
+    </row>
+    <row r="39" ht="65" customHeight="1">
       <c r="A39" s="3" t="n">
         <v>46200</v>
       </c>
@@ -1973,14 +2129,14 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>🏔️ MALAGA J6 — CAP côte : sortie finale</t>
+          <t>🏔️ MALAGA J6 — Finale (descentes à pied)</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
@@ -1997,7 +2153,8 @@
       <c r="H39" s="7" t="inlineStr">
         <is>
           <t>CAMP MALAGA — Jour 6 : Finale légère
-10' EF | 3x [Montée 200m D+ @ Z2-Z3 (138-155 bpm) — descente récup] | 12' RC
+10' EF plat | 3x MONTÉE 200m D+ @ Z2-Z3 (138-155 bpm)
+⚠️ DESCENTES À PIED — jusqu'au bout
 Sortie de clôture — fierté du camp accompli 💪
 D+ cumulé : ~600m</t>
         </is>
@@ -2007,6 +2164,9 @@
       </c>
       <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
+      <c r="L39" s="4" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -2049,6 +2209,7 @@
       <c r="K40" s="4" t="n">
         <v>600</v>
       </c>
+      <c r="L40" s="4" t="n"/>
     </row>
     <row r="41" ht="39" customHeight="1">
       <c r="A41" s="3" t="n">
@@ -2092,6 +2253,7 @@
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="n"/>
       <c r="K41" s="4" t="n"/>
+      <c r="L41" s="4" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="9" t="n"/>
@@ -2103,7 +2265,7 @@
       <c r="G42" s="9" t="n"/>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I42" s="9" t="n">
@@ -2113,11 +2275,12 @@
       <c r="K42" s="9" t="n">
         <v>4100</v>
       </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 5 — 29/06 au 05/07/2026</t>
+      <c r="L42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  29/06 → 05/07/2026   |   Retour vélo 30/06 (cadence haute) + CAP plat + Nat WE</t>
         </is>
       </c>
     </row>
@@ -2161,8 +2324,9 @@
       <c r="I44" s="4" t="n"/>
       <c r="J44" s="4" t="n"/>
       <c r="K44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="65" customHeight="1">
+      <c r="L44" s="4" t="n"/>
+    </row>
+    <row r="45" ht="104" customHeight="1">
       <c r="A45" s="3" t="n">
         <v>46203</v>
       </c>
@@ -2171,14 +2335,14 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>🚴 PREMIER VÉLO — reprise douce Z2</t>
+          <t>🚴 PREMIER VÉLO — cadence haute UNIQUEMENT</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
@@ -2196,9 +2360,12 @@
         <is>
           <t>RETOUR VÉLO après 7 semaines !
 55' Z2 très facile (120-133 bpm)
-Cadence très souple 82-87 rpm — ne pas forcer
-Écouter les sensations — jambes potentiellement très rouillées
-Pas d'intensité — juste tourner les jambes</t>
+PROTOCOLE GENOU :
+  · Cadence HAUTE : 90-95 rpm minimum — réduit la pression sur le genou
+  · Selle légèrement plus haute qu'habitude (1-2 cm)
+  · ZÉRO force — ZÉRO basse cadence pendant 2 semaines
+  · Plateau facile — résistance minimale
+Écouter les sensations du genou</t>
         </is>
       </c>
       <c r="I45" s="4" t="n"/>
@@ -2206,6 +2373,9 @@
         <v>25</v>
       </c>
       <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -2216,14 +2386,14 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>EF légère post-Malaga</t>
+          <t>EF légère post-Malaga — plat</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
@@ -2239,8 +2409,8 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>32' EF Z2 (120-133 bpm) — reprise douce
-Post-camp Malaga — observer les sensations</t>
+          <t>32' EF Z2 (120-133 bpm) — terrain plat
+Post-camp Malaga — observer les sensations genou</t>
         </is>
       </c>
       <c r="I46" s="4" t="n">
@@ -2248,8 +2418,11 @@
       </c>
       <c r="J46" s="4" t="n"/>
       <c r="K46" s="4" t="n"/>
-    </row>
-    <row r="47" ht="26" customHeight="1">
+      <c r="L46" s="4" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" ht="39" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>46204</v>
       </c>
@@ -2258,14 +2431,14 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C47" s="12" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 — 80'</t>
+          <t>Sortie Z2 — 80' (cadence haute)</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
@@ -2281,8 +2454,9 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>80' Z2 (127-138 bpm) — progression vélo
-Cadence 83-90 rpm | NUTRITION : 40g/h si besoin</t>
+          <t>80' Z2 (127-138 bpm)
+Cadence 90-95 rpm — pas de basse cadence
+NUTRITION : 40g/h si besoin</t>
         </is>
       </c>
       <c r="I47" s="4" t="n"/>
@@ -2290,8 +2464,11 @@
         <v>39</v>
       </c>
       <c r="K47" s="4" t="n"/>
-    </row>
-    <row r="48" ht="26" customHeight="1">
+      <c r="L47" s="4" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="48" ht="52" customHeight="1">
       <c r="A48" s="3" t="n">
         <v>46205</v>
       </c>
@@ -2300,14 +2477,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Vélo force légère — 55'</t>
+          <t>Vélo cadence haute — 55' (pas de force)</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
@@ -2315,7 +2492,7 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G48" s="4" t="n">
@@ -2323,8 +2500,10 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>10' EF | 4x5' basse cadence (62 rpm) @ Z2 — r=3' | 15' RC
-Réactivation musculaire — très progressif</t>
+          <t>10' EF | 4x8' cadence HAUTE 95-100 rpm @ Z2 — r=3' | 15' RC
+PROTOCOLE GENOU : PAS de basse cadence avant 2 semaines sans douleur
+Basse cadence = forte pression genou → contre-indiqué
+Cadence haute = cardio sans pression articulaire</t>
         </is>
       </c>
       <c r="I48" s="4" t="n"/>
@@ -2332,6 +2511,9 @@
         <v>26</v>
       </c>
       <c r="K48" s="4" t="n"/>
+      <c r="L48" s="4" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -2342,14 +2524,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>EF — 30'</t>
+          <t>EF — 30' plat</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
@@ -2365,7 +2547,7 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile</t>
+          <t>30' EF Z2 facile — terrain plat</t>
         </is>
       </c>
       <c r="I49" s="4" t="n">
@@ -2373,6 +2555,9 @@
       </c>
       <c r="J49" s="4" t="n"/>
       <c r="K49" s="4" t="n"/>
+      <c r="L49" s="4" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="A50" s="3" t="n">
@@ -2383,14 +2568,14 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>EF + strides — 35'</t>
+          <t>EF + strides — 35' plat</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
@@ -2407,7 +2592,7 @@
       <c r="H50" s="7" t="inlineStr">
         <is>
           <t>30' EF Z2 | 4x20'' strides en fin
-Foncier progressif</t>
+Foncier progressif — terrain plat</t>
         </is>
       </c>
       <c r="I50" s="4" t="n">
@@ -2415,6 +2600,9 @@
       </c>
       <c r="J50" s="4" t="n"/>
       <c r="K50" s="4" t="n"/>
+      <c r="L50" s="4" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="51" ht="39" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -2425,7 +2613,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2449,8 +2637,8 @@
       <c r="H51" s="7" t="inlineStr">
         <is>
           <t>100' Z2 (127-138 bpm) — première vraie longue vélo
-Z2 pur — pas de blocs encore
-NUTRITION : 40g/h | Cadence 83-90 rpm</t>
+Z2 pur — cadence 90-95 rpm — pas de blocs
+NUTRITION : 40g/h | Selle position genou OK</t>
         </is>
       </c>
       <c r="I51" s="4" t="n"/>
@@ -2458,6 +2646,9 @@
         <v>49</v>
       </c>
       <c r="K51" s="4" t="n"/>
+      <c r="L51" s="4" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -2499,6 +2690,7 @@
       <c r="K52" s="4" t="n">
         <v>1500</v>
       </c>
+      <c r="L52" s="4" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="3" t="n">
@@ -2540,8 +2732,9 @@
       <c r="K53" s="4" t="n">
         <v>1500</v>
       </c>
-    </row>
-    <row r="54" ht="26" customHeight="1">
+      <c r="L53" s="4" t="n"/>
+    </row>
+    <row r="54" ht="52" customHeight="1">
       <c r="A54" s="3" t="n">
         <v>46208</v>
       </c>
@@ -2550,14 +2743,14 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 62'</t>
+          <t>Sortie longue Z2 — 62' (plat/vallonné doux)</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
@@ -2574,7 +2767,9 @@
       <c r="H54" s="7" t="inlineStr">
         <is>
           <t>62' Z2 (127-138 bpm) — foncier CAP
-Allure conversationnelle</t>
+Allure conversationnelle
+PROTOCOLE GENOU : plat ou légèrement vallonné
+Éviter les descentes raides — pentes douces uniquement</t>
         </is>
       </c>
       <c r="I54" s="4" t="n">
@@ -2582,6 +2777,9 @@
       </c>
       <c r="J54" s="4" t="n"/>
       <c r="K54" s="4" t="n"/>
+      <c r="L54" s="4" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="9" t="n"/>
@@ -2593,7 +2791,7 @@
       <c r="G55" s="9" t="n"/>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I55" s="9" t="n">
@@ -2605,11 +2803,12 @@
       <c r="K55" s="9" t="n">
         <v>3000</v>
       </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 6 — 06/07 au 12/07/2026</t>
+      <c r="L55" s="9" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  06/07 → 12/07/2026   |   Build — Vélo + CAP + Nat WE 11-12 juil</t>
         </is>
       </c>
     </row>
@@ -2653,6 +2852,7 @@
       <c r="I57" s="4" t="n"/>
       <c r="J57" s="4" t="n"/>
       <c r="K57" s="4" t="n"/>
+      <c r="L57" s="4" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -2663,7 +2863,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C58" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2686,7 +2886,7 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>42' Z2 récup — cadence souple</t>
+          <t>42' Z2 récup — cadence souple 90-95 rpm</t>
         </is>
       </c>
       <c r="I58" s="4" t="n"/>
@@ -2694,6 +2894,9 @@
         <v>19</v>
       </c>
       <c r="K58" s="4" t="n"/>
+      <c r="L58" s="4" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="59" ht="52" customHeight="1">
       <c r="A59" s="3" t="n">
@@ -2704,7 +2907,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2728,9 +2931,9 @@
       <c r="H59" s="7" t="inlineStr">
         <is>
           <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
-Première qualité — FC cible 147-153 bpm
-Ne pas dépasser 155 bpm — progressif
-4x20'' strides en fin</t>
+FC cible : 147-153 bpm — ne pas dépasser 155 bpm
+4x20'' strides en fin
+Terrain plat ou très légèrement ondulé</t>
         </is>
       </c>
       <c r="I59" s="4" t="n">
@@ -2738,6 +2941,9 @@
       </c>
       <c r="J59" s="4" t="n"/>
       <c r="K59" s="4" t="n"/>
+      <c r="L59" s="4" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="60" ht="26" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -2748,7 +2954,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
+      <c r="C60" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2771,7 +2977,7 @@
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>90' Z2 (127-138 bpm) | Cadence 85-90 rpm
+          <t>90' Z2 (127-138 bpm) | Cadence 88-93 rpm
 NUTRITION : 42g/h</t>
         </is>
       </c>
@@ -2780,8 +2986,11 @@
         <v>44</v>
       </c>
       <c r="K60" s="4" t="n"/>
-    </row>
-    <row r="61" ht="18" customHeight="1">
+      <c r="L60" s="4" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" ht="78" customHeight="1">
       <c r="A61" s="3" t="n">
         <v>46212</v>
       </c>
@@ -2790,14 +2999,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C61" s="12" t="inlineStr">
+      <c r="C61" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Force vélo — 65'</t>
+          <t>Vélo cadence mixte — 65'</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
@@ -2809,11 +3018,16 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>10' EF | 5x5' basse cadence (60 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm | 10' RC</t>
+          <t>10' EF
+SI genou symptôme-free depuis 1 semaine :
+  4x5' basse cadence (65 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm
+SINON :
+  6x8' cadence haute 92-97 rpm @ Z2 — r=2'
+Toujours écouter le genou</t>
         </is>
       </c>
       <c r="I61" s="4" t="n"/>
@@ -2821,6 +3035,9 @@
         <v>31</v>
       </c>
       <c r="K61" s="4" t="n"/>
+      <c r="L61" s="4" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="3" t="n">
@@ -2831,7 +3048,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C62" s="11" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2854,7 +3071,7 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile</t>
+          <t>30' EF Z2 facile — plat</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
@@ -2862,6 +3079,9 @@
       </c>
       <c r="J62" s="4" t="n"/>
       <c r="K62" s="4" t="n"/>
+      <c r="L62" s="4" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -2872,7 +3092,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2896,7 +3116,7 @@
       <c r="H63" s="7" t="inlineStr">
         <is>
           <t>12' EF | 2x15' Z3 (148-156 bpm) — r=3' | 12' RC
-FC cible : 148-156 bpm — régulier</t>
+FC cible : 148-156 bpm — terrain plat</t>
         </is>
       </c>
       <c r="I63" s="4" t="n">
@@ -2904,6 +3124,9 @@
       </c>
       <c r="J63" s="4" t="n"/>
       <c r="K63" s="4" t="n"/>
+      <c r="L63" s="4" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="64" ht="26" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -2914,7 +3137,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C64" s="12" t="inlineStr">
+      <c r="C64" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2938,7 +3161,7 @@
       <c r="H64" s="7" t="inlineStr">
         <is>
           <t>120' Z2 (127-140 bpm) | 2x18' Z3 inclus — r=10'
-NUTRITION : 45g/h | Cadence 85-92 rpm</t>
+NUTRITION : 45g/h | Cadence 88-93 rpm</t>
         </is>
       </c>
       <c r="I64" s="4" t="n"/>
@@ -2946,6 +3169,9 @@
         <v>59</v>
       </c>
       <c r="K64" s="4" t="n"/>
+      <c r="L64" s="4" t="n">
+        <v>157</v>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="3" t="n">
@@ -2987,6 +3213,7 @@
       <c r="K65" s="4" t="n">
         <v>1700</v>
       </c>
+      <c r="L65" s="4" t="n"/>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -3028,8 +3255,9 @@
       <c r="K66" s="4" t="n">
         <v>1700</v>
       </c>
-    </row>
-    <row r="67" ht="26" customHeight="1">
+      <c r="L66" s="4" t="n"/>
+    </row>
+    <row r="67" ht="39" customHeight="1">
       <c r="A67" s="3" t="n">
         <v>46215</v>
       </c>
@@ -3038,14 +3266,14 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C67" s="11" t="inlineStr">
+      <c r="C67" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 75'</t>
+          <t>Sortie longue Z2 — 75' (plat/vallonné doux)</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
@@ -3062,7 +3290,8 @@
       <c r="H67" s="7" t="inlineStr">
         <is>
           <t>75' Z2 (127-140 bpm) — foncier
-Allure conversationnelle</t>
+Allure conversationnelle
+Genou : éviter les descentes raides — terrain plat/légèrement vallonné</t>
         </is>
       </c>
       <c r="I67" s="4" t="n">
@@ -3070,6 +3299,9 @@
       </c>
       <c r="J67" s="4" t="n"/>
       <c r="K67" s="4" t="n"/>
+      <c r="L67" s="4" t="n">
+        <v>64</v>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="9" t="n"/>
@@ -3081,7 +3313,7 @@
       <c r="G68" s="9" t="n"/>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I68" s="9" t="n">
@@ -3093,11 +3325,12 @@
       <c r="K68" s="9" t="n">
         <v>3400</v>
       </c>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 7 — 13/07 au 19/07/2026</t>
+      <c r="L68" s="9" t="n"/>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  13/07 → 19/07/2026   |   Build pic pré-vacances — Vélo + CAP + Nat WE 18-19</t>
         </is>
       </c>
     </row>
@@ -3141,6 +3374,7 @@
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="4" t="n"/>
       <c r="K70" s="4" t="n"/>
+      <c r="L70" s="4" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="3" t="n">
@@ -3151,7 +3385,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3174,7 +3408,7 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>42' Z2 récup</t>
+          <t>42' Z2 récup — cadence 90-95 rpm</t>
         </is>
       </c>
       <c r="I71" s="4" t="n"/>
@@ -3182,8 +3416,11 @@
         <v>19</v>
       </c>
       <c r="K71" s="4" t="n"/>
-    </row>
-    <row r="72" ht="78" customHeight="1">
+      <c r="L71" s="4" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="72" ht="91" customHeight="1">
       <c r="A72" s="3" t="n">
         <v>46217</v>
       </c>
@@ -3192,7 +3429,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
+      <c r="C72" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3220,7 +3457,8 @@
   Rép 1-2 : 83-84% FCmax → FC 161-164 bpm
   Rép 3-4 : 85% FCmax → FC 164-166 bpm
 r=1'30 — FC sous 145 bpm
-10' RC</t>
+10' RC
+Terrain plat</t>
         </is>
       </c>
       <c r="I72" s="4" t="n">
@@ -3228,6 +3466,9 @@
       </c>
       <c r="J72" s="4" t="n"/>
       <c r="K72" s="4" t="n"/>
+      <c r="L72" s="4" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -3238,7 +3479,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C73" s="12" t="inlineStr">
+      <c r="C73" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3270,8 +3511,11 @@
         <v>51</v>
       </c>
       <c r="K73" s="4" t="n"/>
-    </row>
-    <row r="74" ht="18" customHeight="1">
+      <c r="L73" s="4" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="74" ht="65" customHeight="1">
       <c r="A74" s="3" t="n">
         <v>46219</v>
       </c>
@@ -3280,14 +3524,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C74" s="12" t="inlineStr">
+      <c r="C74" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Force vélo — 70'</t>
+          <t>Force vélo — 70' (si asymptomatique)</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
@@ -3303,7 +3547,11 @@
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>10' EF | 5x6' basse cadence (58 rpm) @ Z2-Z3 — r=3' + 2x5' cadence 100 rpm | 10' RC</t>
+          <t>10' EF
+SI symptôme-free depuis 2 semaines → programme normal :
+  5x6' basse cadence (60 rpm) @ Z2-Z3 — r=3' + 2x5' cadence 100 rpm
+SI encore sensible → cadence haute uniquement :
+  6x8' cadence 92-97 rpm @ Z2 — r=2'</t>
         </is>
       </c>
       <c r="I74" s="4" t="n"/>
@@ -3311,6 +3559,9 @@
         <v>33</v>
       </c>
       <c r="K74" s="4" t="n"/>
+      <c r="L74" s="4" t="n">
+        <v>112</v>
+      </c>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -3321,7 +3572,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C75" s="11" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3344,7 +3595,7 @@
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>32' EF Z2 facile</t>
+          <t>32' EF Z2 facile — plat</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -3352,6 +3603,9 @@
       </c>
       <c r="J75" s="4" t="n"/>
       <c r="K75" s="4" t="n"/>
+      <c r="L75" s="4" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="76" ht="26" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -3362,7 +3616,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C76" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3386,7 +3640,7 @@
       <c r="H76" s="7" t="inlineStr">
         <is>
           <t>12' EF | 2x18' Z3 (150-158 bpm) — r=3' | 12' RC
-FC cible : 150-158 bpm</t>
+FC cible : 150-158 bpm — terrain plat</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
@@ -3394,6 +3648,9 @@
       </c>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
+      <c r="L76" s="4" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="77" ht="39" customHeight="1">
       <c r="A77" s="3" t="n">
@@ -3404,7 +3661,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C77" s="12" t="inlineStr">
+      <c r="C77" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3427,7 +3684,7 @@
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>140' Z2 (127-140 bpm) — PIC avant les vacances
+          <t>140' Z2 (127-140 bpm) — PIC avant vacances
 2x22' Z3 inclus — r=10'
 NUTRITION : 48g/h | Cadence 85-93 rpm</t>
         </is>
@@ -3437,8 +3694,11 @@
         <v>68</v>
       </c>
       <c r="K77" s="4" t="n"/>
-    </row>
-    <row r="78" ht="26" customHeight="1">
+      <c r="L77" s="4" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="n">
         <v>46221</v>
       </c>
@@ -3470,8 +3730,7 @@
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>4x50 facile | 10x50 éducatifs | 3x300 continu | 300 retour — 1 800 m
-Dernière nat structurée avant vacances</t>
+          <t>4x50 facile | 10x50 éducatifs | 3x300 continu | 300 retour — 1 800 m</t>
         </is>
       </c>
       <c r="I78" s="4" t="n"/>
@@ -3479,6 +3738,7 @@
       <c r="K78" s="4" t="n">
         <v>1800</v>
       </c>
+      <c r="L78" s="4" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -3520,8 +3780,9 @@
       <c r="K79" s="4" t="n">
         <v>1800</v>
       </c>
-    </row>
-    <row r="80" ht="26" customHeight="1">
+      <c r="L79" s="4" t="n"/>
+    </row>
+    <row r="80" ht="39" customHeight="1">
       <c r="A80" s="3" t="n">
         <v>46222</v>
       </c>
@@ -3530,7 +3791,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C80" s="11" t="inlineStr">
+      <c r="C80" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3554,7 +3815,8 @@
       <c r="H80" s="7" t="inlineStr">
         <is>
           <t>82' Z2 (127-140 bpm) — pic avant Italie
-Allure conversationnelle</t>
+Allure conversationnelle
+Genou : toujours terrain plat/légèrement vallonné — descentes douces</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
@@ -3562,6 +3824,9 @@
       </c>
       <c r="J80" s="4" t="n"/>
       <c r="K80" s="4" t="n"/>
+      <c r="L80" s="4" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="9" t="n"/>
@@ -3573,7 +3838,7 @@
       <c r="G81" s="9" t="n"/>
       <c r="H81" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I81" s="9" t="n">
@@ -3585,11 +3850,12 @@
       <c r="K81" s="9" t="n">
         <v>3600</v>
       </c>
-    </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 8 — 20/07 au 26/07/2026</t>
+      <c r="L81" s="9" t="n"/>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  20/07 → 22/07/2026   |   Transition — dernière semaine avant vacances</t>
         </is>
       </c>
     </row>
@@ -3633,6 +3899,7 @@
       <c r="I83" s="4" t="n"/>
       <c r="J83" s="4" t="n"/>
       <c r="K83" s="4" t="n"/>
+      <c r="L83" s="4" t="n"/>
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -3643,7 +3910,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr">
+      <c r="C84" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3675,6 +3942,9 @@
         <v>29</v>
       </c>
       <c r="K84" s="4" t="n"/>
+      <c r="L84" s="4" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -3685,7 +3955,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
+      <c r="C85" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3716,6 +3986,9 @@
       </c>
       <c r="J85" s="4" t="n"/>
       <c r="K85" s="4" t="n"/>
+      <c r="L85" s="4" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="3" t="n">
@@ -3726,7 +3999,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C86" s="12" t="inlineStr">
+      <c r="C86" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3757,96 +4030,46 @@
         <v>32</v>
       </c>
       <c r="K86" s="4" t="n"/>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="3" t="n">
-        <v>46226</v>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>Jeudi</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G87" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H87" s="7" t="inlineStr">
-        <is>
-          <t>🇮🇹 Voyage Luxembourg→Florence — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I87" s="4" t="n"/>
-      <c r="J87" s="4" t="n"/>
-      <c r="K87" s="4" t="n"/>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="3" t="n">
-        <v>46227</v>
-      </c>
-      <c r="B88" s="4" t="inlineStr">
-        <is>
-          <t>Vendredi</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D88" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G88" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H88" s="7" t="inlineStr">
-        <is>
-          <t>🇮🇹 Florence (excursion Sienne) — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I88" s="4" t="n"/>
-      <c r="J88" s="4" t="n"/>
-      <c r="K88" s="4" t="n"/>
+      <c r="L86" s="4" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="9" t="n"/>
+      <c r="B87" s="9" t="n"/>
+      <c r="C87" s="9" t="n"/>
+      <c r="D87" s="9" t="n"/>
+      <c r="E87" s="9" t="n"/>
+      <c r="F87" s="9" t="n"/>
+      <c r="G87" s="9" t="n"/>
+      <c r="H87" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PÉRIODE</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J87" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="K87" s="9" t="n"/>
+      <c r="L87" s="9" t="n"/>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  23/07 → 09/08/2026   |   🇮🇹🇬🇷 VACANCES Italie + Grèce — ZÉRO SÉANCE</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="3" t="n">
-        <v>46228</v>
+        <v>46226</v>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Samedi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -3874,20 +4097,21 @@
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>🇮🇹 Florence — ZÉRO SÉANCE</t>
+          <t>🇮🇹 Voyage Luxembourg→Florence — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I89" s="4" t="n"/>
       <c r="J89" s="4" t="n"/>
       <c r="K89" s="4" t="n"/>
+      <c r="L89" s="4" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="3" t="n">
-        <v>46229</v>
+        <v>46227</v>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -3915,40 +4139,97 @@
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>🇮🇹 Florence→Rome (train 19h45) — ZÉRO SÉANCE</t>
+          <t>🇮🇹 Florence (excursion Sienne) — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I90" s="4" t="n"/>
       <c r="J90" s="4" t="n"/>
       <c r="K90" s="4" t="n"/>
-    </row>
-    <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="9" t="n"/>
-      <c r="B91" s="9" t="n"/>
-      <c r="C91" s="9" t="n"/>
-      <c r="D91" s="9" t="n"/>
-      <c r="E91" s="9" t="n"/>
-      <c r="F91" s="9" t="n"/>
-      <c r="G91" s="9" t="n"/>
-      <c r="H91" s="10" t="inlineStr">
-        <is>
-          <t>Total semaine</t>
-        </is>
-      </c>
-      <c r="I91" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="J91" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="K91" s="9" t="n"/>
+      <c r="L90" s="4" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="3" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>🇮🇹 Florence — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I91" s="4" t="n"/>
+      <c r="J91" s="4" t="n"/>
+      <c r="K91" s="4" t="n"/>
+      <c r="L91" s="4" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 9 — 27/07 au 02/08/2026</t>
-        </is>
-      </c>
+      <c r="A92" s="3" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>🇮🇹 Florence→Rome — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
+      <c r="L92" s="4" t="n"/>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -3990,6 +4271,7 @@
       <c r="I93" s="4" t="n"/>
       <c r="J93" s="4" t="n"/>
       <c r="K93" s="4" t="n"/>
+      <c r="L93" s="4" t="n"/>
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -4031,6 +4313,7 @@
       <c r="I94" s="4" t="n"/>
       <c r="J94" s="4" t="n"/>
       <c r="K94" s="4" t="n"/>
+      <c r="L94" s="4" t="n"/>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="3" t="n">
@@ -4072,6 +4355,7 @@
       <c r="I95" s="4" t="n"/>
       <c r="J95" s="4" t="n"/>
       <c r="K95" s="4" t="n"/>
+      <c r="L95" s="4" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -4113,6 +4397,7 @@
       <c r="I96" s="4" t="n"/>
       <c r="J96" s="4" t="n"/>
       <c r="K96" s="4" t="n"/>
+      <c r="L96" s="4" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -4154,6 +4439,7 @@
       <c r="I97" s="4" t="n"/>
       <c r="J97" s="4" t="n"/>
       <c r="K97" s="4" t="n"/>
+      <c r="L97" s="4" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="3" t="n">
@@ -4195,6 +4481,7 @@
       <c r="I98" s="4" t="n"/>
       <c r="J98" s="4" t="n"/>
       <c r="K98" s="4" t="n"/>
+      <c r="L98" s="4" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -4236,38 +4523,99 @@
       <c r="I99" s="4" t="n"/>
       <c r="J99" s="4" t="n"/>
       <c r="K99" s="4" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="9" t="n"/>
-      <c r="B100" s="9" t="n"/>
-      <c r="C100" s="9" t="n"/>
-      <c r="D100" s="9" t="n"/>
-      <c r="E100" s="9" t="n"/>
-      <c r="F100" s="9" t="n"/>
-      <c r="G100" s="9" t="n"/>
-      <c r="H100" s="10" t="inlineStr">
-        <is>
-          <t>Total semaine</t>
-        </is>
-      </c>
-      <c r="I100" s="9" t="n"/>
-      <c r="J100" s="9" t="n"/>
-      <c r="K100" s="9" t="n"/>
+      <c r="L99" s="4" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" s="7" t="inlineStr">
+        <is>
+          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="n"/>
+      <c r="J100" s="4" t="n"/>
+      <c r="K100" s="4" t="n"/>
+      <c r="L100" s="4" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 10 — 03/08 au 09/08/2026</t>
-        </is>
-      </c>
+      <c r="A101" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="4" t="n"/>
+      <c r="K101" s="4" t="n"/>
+      <c r="L101" s="4" t="n"/>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="3" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Lundi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
@@ -4301,14 +4649,15 @@
       <c r="I102" s="4" t="n"/>
       <c r="J102" s="4" t="n"/>
       <c r="K102" s="4" t="n"/>
+      <c r="L102" s="4" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="3" t="n">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Mardi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
@@ -4342,14 +4691,15 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
       <c r="K103" s="4" t="n"/>
+      <c r="L103" s="4" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="3" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
@@ -4383,14 +4733,15 @@
       <c r="I104" s="4" t="n"/>
       <c r="J104" s="4" t="n"/>
       <c r="K104" s="4" t="n"/>
+      <c r="L104" s="4" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="3" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Samedi</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
@@ -4424,14 +4775,15 @@
       <c r="I105" s="4" t="n"/>
       <c r="J105" s="4" t="n"/>
       <c r="K105" s="4" t="n"/>
+      <c r="L105" s="4" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="3" t="n">
-        <v>46241</v>
+        <v>46243</v>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Vendredi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
@@ -4459,225 +4811,246 @@
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
+          <t>🇬🇷→🇱🇺 Retour Thessalonique→Luxembourg — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I106" s="4" t="n"/>
       <c r="J106" s="4" t="n"/>
       <c r="K106" s="4" t="n"/>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="3" t="n">
-        <v>46242</v>
-      </c>
-      <c r="B107" s="4" t="inlineStr">
-        <is>
-          <t>Samedi</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
+      <c r="L106" s="4" t="n"/>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="9" t="n"/>
+      <c r="B107" s="9" t="n"/>
+      <c r="C107" s="9" t="n"/>
+      <c r="D107" s="9" t="n"/>
+      <c r="E107" s="9" t="n"/>
+      <c r="F107" s="9" t="n"/>
+      <c r="G107" s="9" t="n"/>
+      <c r="H107" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PÉRIODE</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="n"/>
+      <c r="J107" s="9" t="n"/>
+      <c r="K107" s="9" t="n"/>
+      <c r="L107" s="9" t="n"/>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  10/08 → 16/08/2026   |   ⚡ REPRISE CRITIQUE J-21 plan IM | Nat WE 15-16 août</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="91" customHeight="1">
+      <c r="A109" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="D107" s="6" t="inlineStr">
+      <c r="D109" s="6" t="inlineStr">
         <is>
           <t>OFF / Repos</t>
         </is>
       </c>
-      <c r="E107" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F107" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G107" s="4" t="n">
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H107" s="7" t="inlineStr">
-        <is>
-          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I107" s="4" t="n"/>
-      <c r="J107" s="4" t="n"/>
-      <c r="K107" s="4" t="n"/>
-    </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="3" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t>Dimanche</t>
-        </is>
-      </c>
-      <c r="C108" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E108" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F108" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G108" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H108" s="7" t="inlineStr">
-        <is>
-          <t>🇬🇷→🇱🇺 Retour Thessalonique→Luxembourg — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I108" s="4" t="n"/>
-      <c r="J108" s="4" t="n"/>
-      <c r="K108" s="4" t="n"/>
-    </row>
-    <row r="109" ht="15" customHeight="1">
-      <c r="A109" s="9" t="n"/>
-      <c r="B109" s="9" t="n"/>
-      <c r="C109" s="9" t="n"/>
-      <c r="D109" s="9" t="n"/>
-      <c r="E109" s="9" t="n"/>
-      <c r="F109" s="9" t="n"/>
-      <c r="G109" s="9" t="n"/>
-      <c r="H109" s="10" t="inlineStr">
-        <is>
-          <t>Total semaine</t>
-        </is>
-      </c>
-      <c r="I109" s="9" t="n"/>
-      <c r="J109" s="9" t="n"/>
-      <c r="K109" s="9" t="n"/>
-    </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 11 — 10/08 au 16/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="26" customHeight="1">
+      <c r="H109" s="7" t="inlineStr">
+        <is>
+          <t>Repos — récup voyage retour Grèce
+J-21 plan Ironman — reprise ultra-progressive
+STRATÉGIE 3 SEMAINES :
+Sem 1 (10-16) : RPE max 5/10 — reconstruire les automatismes
+Sem 2 (17-23) : Luxembourg vélo → boost cardiovasculaire clé
+Sem 3 (24-30) : Volume -20% — arriver FRAIS le 31 août</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="4" t="n"/>
+      <c r="K109" s="4" t="n"/>
+      <c r="L109" s="4" t="n"/>
+    </row>
+    <row r="110" ht="52" customHeight="1">
+      <c r="A110" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C110" s="12" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>EF reprise — post-vacances plat</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>Z1-Z2</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H110" s="7" t="inlineStr">
+        <is>
+          <t>35' EF Z2 (120-133 bpm) — reprise très douce
+18 jours sans séance — ne pas forcer
+Terrain plat — surveiller le genou
+Marche-course si besoin</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J110" s="4" t="n"/>
+      <c r="K110" s="4" t="n"/>
+      <c r="L110" s="4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="111" ht="39" customHeight="1">
       <c r="A111" s="3" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Lundi</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C111" s="16" t="inlineStr">
+        <is>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E111" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Vélo reprise Z2 — 48' (cadence haute)</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>48</v>
       </c>
       <c r="F111" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H111" s="7" t="inlineStr">
         <is>
-          <t>Repos — récup voyage retour Grèce
-J-21 plan Ironman — reprise ultra-progressive</t>
+          <t>48' Z2 — reprendre les jambes vélo
+Cadence 90-95 rpm — jamais &gt; Z2
+Genou : cadence haute encore obligatoire</t>
         </is>
       </c>
       <c r="I111" s="4" t="n"/>
-      <c r="J111" s="4" t="n"/>
+      <c r="J111" s="4" t="n">
+        <v>22</v>
+      </c>
       <c r="K111" s="4" t="n"/>
+      <c r="L111" s="4" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="112" ht="39" customHeight="1">
       <c r="A112" s="3" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C112" s="11" t="inlineStr">
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="inlineStr">
+        <is>
+          <t>Vélo</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>Sortie Z2 + SS reprise — 115'</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>Z2-Z3</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H112" s="7" t="inlineStr">
+        <is>
+          <t>20' EF | 2x20' SS @ 81% FTP — r=6' | Z2 reste | 15' RC
+Reprise progressive — intensité réduite
+NUTRITION : 43g/h</t>
+        </is>
+      </c>
+      <c r="I112" s="4" t="n"/>
+      <c r="J112" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="K112" s="4" t="n"/>
+      <c r="L112" s="4" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
-        <is>
-          <t>EF reprise — post-vacances</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="F112" s="6" t="inlineStr">
-        <is>
-          <t>Z1-Z2</t>
-        </is>
-      </c>
-      <c r="G112" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H112" s="7" t="inlineStr">
-        <is>
-          <t>35' EF Z2 (120-133 bpm) — reprise très douce
-18 jours sans séance — ne pas forcer
-Marche-course si besoin — écouter le corps</t>
-        </is>
-      </c>
-      <c r="I112" s="4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="J112" s="4" t="n"/>
-      <c r="K112" s="4" t="n"/>
-    </row>
-    <row r="113" ht="39" customHeight="1">
-      <c r="A113" s="3" t="n">
-        <v>46245</v>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C113" s="12" t="inlineStr">
-        <is>
-          <t>Vélo</t>
-        </is>
-      </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Vélo reprise Z2 — 48'</t>
+          <t>EF — 33' plat</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
@@ -4689,38 +5062,39 @@
       </c>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>48' Z2 — reprendre les jambes vélo
-Cadence souple — jamais &gt; Z2
-Sensations premières</t>
-        </is>
-      </c>
-      <c r="I113" s="4" t="n"/>
-      <c r="J113" s="4" t="n">
-        <v>22</v>
-      </c>
+          <t>33' EF Z2 facile — terrain plat</t>
+        </is>
+      </c>
+      <c r="I113" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J113" s="4" t="n"/>
       <c r="K113" s="4" t="n"/>
-    </row>
-    <row r="114" ht="39" customHeight="1">
+      <c r="L113" s="4" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="114" ht="52" customHeight="1">
       <c r="A114" s="3" t="n">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Mercredi</t>
-        </is>
-      </c>
-      <c r="C114" s="12" t="inlineStr">
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C114" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 + SS reprise — 115'</t>
+          <t>Force légère — 60' (si asymptomatique)</t>
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
@@ -4728,456 +5102,394 @@
         </is>
       </c>
       <c r="G114" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H114" s="7" t="inlineStr">
         <is>
-          <t>20' EF | 2x20' SS @ 81% FTP — r=6' | Z2 reste | 15' RC
-Reprise progressive des blocs — intensité réduite
-NUTRITION : 43g/h</t>
+          <t>10' EF
+SI genou asymptomatique :
+  4x6' basse cadence (60 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm
+SINON : cadence haute 92-97 rpm uniquement</t>
         </is>
       </c>
       <c r="I114" s="4" t="n"/>
       <c r="J114" s="4" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="K114" s="4" t="n"/>
-    </row>
-    <row r="115" ht="18" customHeight="1">
+      <c r="L114" s="4" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="115" ht="39" customHeight="1">
       <c r="A115" s="3" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Jeudi</t>
-        </is>
-      </c>
-      <c r="C115" s="11" t="inlineStr">
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>EF — 33'</t>
+          <t>Tempo très léger — 2x12'</t>
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="G115" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H115" s="7" t="inlineStr">
         <is>
-          <t>33' EF Z2 facile</t>
+          <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
+Post-vacances — très contrôlé
+FC cible : 147-153 bpm max — terrain plat</t>
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="J115" s="4" t="n"/>
       <c r="K115" s="4" t="n"/>
-    </row>
-    <row r="116" ht="18" customHeight="1">
+      <c r="L115" s="4" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="116" ht="26" customHeight="1">
       <c r="A116" s="3" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Vendredi</t>
-        </is>
-      </c>
-      <c r="C116" s="12" t="inlineStr">
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C116" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>Force légère — 60'</t>
+          <t>Sortie longue Z2 — 140'</t>
         </is>
       </c>
       <c r="E116" s="4" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="F116" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H116" s="7" t="inlineStr">
         <is>
-          <t>10' EF | 4x6' basse cadence (60 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm | 10' RC</t>
+          <t>140' Z2 (127-140 bpm) | 2x22' Z3 inclus — r=10'
+NUTRITION : 47g/h | Cadence 85-92 rpm</t>
         </is>
       </c>
       <c r="I116" s="4" t="n"/>
       <c r="J116" s="4" t="n">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="K116" s="4" t="n"/>
-    </row>
-    <row r="117" ht="39" customHeight="1">
+      <c r="L116" s="4" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Vendredi</t>
-        </is>
-      </c>
-      <c r="C117" s="11" t="inlineStr">
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>🏊 Natation technique — 1600m</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H117" s="7" t="inlineStr">
+        <is>
+          <t>4x50 facile | 10x50 éducatifs | 3x250 continu | 350 retour — 1 600 m</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="n"/>
+      <c r="J117" s="4" t="n"/>
+      <c r="K117" s="4" t="n">
+        <v>1600</v>
+      </c>
+      <c r="L117" s="4" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>Natation</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>🏊 Natation endurance — 1600m</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H118" s="7" t="inlineStr">
+        <is>
+          <t>200 EF | 2x600 continu (r=25'') | 200 retour — 1 600 m</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n"/>
+      <c r="K118" s="4" t="n">
+        <v>1600</v>
+      </c>
+      <c r="L118" s="4" t="n"/>
+    </row>
+    <row r="119" ht="39" customHeight="1">
+      <c r="A119" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>Tempo très léger — 2x12'</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="F117" s="6" t="inlineStr">
-        <is>
-          <t>Z3</t>
-        </is>
-      </c>
-      <c r="G117" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H117" s="7" t="inlineStr">
-        <is>
-          <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
-Post-vacances — très contrôlé
-FC cible : 147-153 bpm max</t>
-        </is>
-      </c>
-      <c r="I117" s="4" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J117" s="4" t="n"/>
-      <c r="K117" s="4" t="n"/>
-    </row>
-    <row r="118" ht="39" customHeight="1">
-      <c r="A118" s="3" t="n">
-        <v>46249</v>
-      </c>
-      <c r="B118" s="4" t="inlineStr">
-        <is>
-          <t>Samedi</t>
-        </is>
-      </c>
-      <c r="C118" s="12" t="inlineStr">
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>Sortie longue Z2 — 78' (plat/vallonné)</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H119" s="7" t="inlineStr">
+        <is>
+          <t>78' Z2 (127-140 bpm) — foncier solide
+Allure conversationnelle
+Genou : terrain plat ou légèrement vallonné</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="J119" s="4" t="n"/>
+      <c r="K119" s="4" t="n"/>
+      <c r="L119" s="4" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="120" ht="15" customHeight="1">
+      <c r="A120" s="9" t="n"/>
+      <c r="B120" s="9" t="n"/>
+      <c r="C120" s="9" t="n"/>
+      <c r="D120" s="9" t="n"/>
+      <c r="E120" s="9" t="n"/>
+      <c r="F120" s="9" t="n"/>
+      <c r="G120" s="9" t="n"/>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PÉRIODE</t>
+        </is>
+      </c>
+      <c r="I120" s="9" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="J120" s="9" t="n">
+        <v>174</v>
+      </c>
+      <c r="K120" s="9" t="n">
+        <v>3200</v>
+      </c>
+      <c r="L120" s="9" t="n"/>
+    </row>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  17/08 → 20/08/2026   |   Build final 17-20 août</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H122" s="7" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="n"/>
+      <c r="J122" s="4" t="n"/>
+      <c r="K122" s="4" t="n"/>
+      <c r="L122" s="4" t="n"/>
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C123" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>Sortie longue Z2 — 140'</t>
-        </is>
-      </c>
-      <c r="E118" s="4" t="n">
-        <v>140</v>
-      </c>
-      <c r="F118" s="6" t="inlineStr">
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>Vélo récup Z2 — 42'</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G118" s="4" t="n">
+      <c r="G123" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H123" s="7" t="inlineStr">
+        <is>
+          <t>42' Z2 récup — cadence 90-95 rpm</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="n"/>
+      <c r="J123" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K123" s="4" t="n"/>
+      <c r="L123" s="4" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="124" ht="91" customHeight="1">
+      <c r="A124" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C124" s="12" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Qualité — 5x2000m progressif</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>Z3-Z4</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H118" s="7" t="inlineStr">
-        <is>
-          <t>140' Z2 (127-140 bpm) | 2x22' Z3 inclus — r=10'
-NUTRITION : 47g/h | Cadence 85-92 rpm
-Reprise du long samedi — signal important</t>
-        </is>
-      </c>
-      <c r="I118" s="4" t="n"/>
-      <c r="J118" s="4" t="n">
-        <v>68</v>
-      </c>
-      <c r="K118" s="4" t="n"/>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="3" t="n">
-        <v>46249</v>
-      </c>
-      <c r="B119" s="4" t="inlineStr">
-        <is>
-          <t>Samedi</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>Natation</t>
-        </is>
-      </c>
-      <c r="D119" s="6" t="inlineStr">
-        <is>
-          <t>🏊 Natation technique — 1600m</t>
-        </is>
-      </c>
-      <c r="E119" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="F119" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G119" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H119" s="7" t="inlineStr">
-        <is>
-          <t>4x50 facile | 10x50 éducatifs | 3x250 continu | 350 retour — 1 600 m</t>
-        </is>
-      </c>
-      <c r="I119" s="4" t="n"/>
-      <c r="J119" s="4" t="n"/>
-      <c r="K119" s="4" t="n">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="3" t="n">
-        <v>46250</v>
-      </c>
-      <c r="B120" s="4" t="inlineStr">
-        <is>
-          <t>Dimanche</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>Natation</t>
-        </is>
-      </c>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>🏊 Natation endurance — 1600m</t>
-        </is>
-      </c>
-      <c r="E120" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="F120" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G120" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H120" s="7" t="inlineStr">
-        <is>
-          <t>200 EF | 2x600 continu (r=25'') | 200 retour — 1 600 m</t>
-        </is>
-      </c>
-      <c r="I120" s="4" t="n"/>
-      <c r="J120" s="4" t="n"/>
-      <c r="K120" s="4" t="n">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="121" ht="26" customHeight="1">
-      <c r="A121" s="3" t="n">
-        <v>46250</v>
-      </c>
-      <c r="B121" s="4" t="inlineStr">
-        <is>
-          <t>Dimanche</t>
-        </is>
-      </c>
-      <c r="C121" s="11" t="inlineStr">
-        <is>
-          <t>Course</t>
-        </is>
-      </c>
-      <c r="D121" s="6" t="inlineStr">
-        <is>
-          <t>Sortie longue Z2 — 78'</t>
-        </is>
-      </c>
-      <c r="E121" s="4" t="n">
-        <v>78</v>
-      </c>
-      <c r="F121" s="6" t="inlineStr">
-        <is>
-          <t>Z2</t>
-        </is>
-      </c>
-      <c r="G121" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H121" s="7" t="inlineStr">
-        <is>
-          <t>78' Z2 (127-140 bpm) — foncier solide
-Allure conversationnelle</t>
-        </is>
-      </c>
-      <c r="I121" s="4" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="J121" s="4" t="n"/>
-      <c r="K121" s="4" t="n"/>
-    </row>
-    <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="9" t="n"/>
-      <c r="B122" s="9" t="n"/>
-      <c r="C122" s="9" t="n"/>
-      <c r="D122" s="9" t="n"/>
-      <c r="E122" s="9" t="n"/>
-      <c r="F122" s="9" t="n"/>
-      <c r="G122" s="9" t="n"/>
-      <c r="H122" s="10" t="inlineStr">
-        <is>
-          <t>Total semaine</t>
-        </is>
-      </c>
-      <c r="I122" s="9" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="J122" s="9" t="n">
-        <v>174</v>
-      </c>
-      <c r="K122" s="9" t="n">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="123" ht="18" customHeight="1">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 12 — 17/08 au 23/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="3" t="n">
-        <v>46251</v>
-      </c>
-      <c r="B124" s="4" t="inlineStr">
-        <is>
-          <t>Lundi</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F124" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G124" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="H124" s="7" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I124" s="4" t="n"/>
-      <c r="J124" s="4" t="n"/>
-      <c r="K124" s="4" t="n"/>
-    </row>
-    <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="3" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B125" s="4" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C125" s="12" t="inlineStr">
-        <is>
-          <t>Vélo</t>
-        </is>
-      </c>
-      <c r="D125" s="6" t="inlineStr">
-        <is>
-          <t>Vélo récup Z2 — 42'</t>
-        </is>
-      </c>
-      <c r="E125" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="F125" s="6" t="inlineStr">
-        <is>
-          <t>Z2</t>
-        </is>
-      </c>
-      <c r="G125" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H125" s="7" t="inlineStr">
-        <is>
-          <t>42' Z2 récup</t>
-        </is>
-      </c>
-      <c r="I125" s="4" t="n"/>
-      <c r="J125" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="K125" s="4" t="n"/>
-    </row>
-    <row r="126" ht="91" customHeight="1">
-      <c r="A126" s="3" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B126" s="4" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C126" s="11" t="inlineStr">
-        <is>
-          <t>Course</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>Qualité — 5x2000m progressif</t>
-        </is>
-      </c>
-      <c r="E126" s="4" t="n">
-        <v>63</v>
-      </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>Z3-Z4</t>
-        </is>
-      </c>
-      <c r="G126" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H126" s="7" t="inlineStr">
         <is>
           <t>12' EF
 5x2000m progressif :
@@ -5185,97 +5497,135 @@
   Rép 2-3 : 83% → FC 161-164 bpm
   Rép 4-5 : 85% → FC 164-166 bpm
 r=1'30 — FC sous 145 bpm
-10' RC</t>
+10' RC — terrain plat</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="J124" s="4" t="n"/>
+      <c r="K124" s="4" t="n"/>
+      <c r="L124" s="4" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="125" ht="26" customHeight="1">
+      <c r="A125" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C125" s="16" t="inlineStr">
+        <is>
+          <t>Vélo</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>Sortie Z2 + SS — 125'</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>Z2-Z3</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H125" s="7" t="inlineStr">
+        <is>
+          <t>20' EF | 2x24' SS @ 84% FTP — r=7' | Z2 reste | 15' RC
+NUTRITION : 48g/h</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="n"/>
+      <c r="J125" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="K125" s="4" t="n"/>
+      <c r="L125" s="4" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="126" ht="18" customHeight="1">
+      <c r="A126" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C126" s="12" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>EF — 30'</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>Z2</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H126" s="7" t="inlineStr">
+        <is>
+          <t>30' EF Z2 — économiser pour Luxembourg vélo</t>
         </is>
       </c>
       <c r="I126" s="4" t="n">
-        <v>12</v>
+        <v>5.5</v>
       </c>
       <c r="J126" s="4" t="n"/>
       <c r="K126" s="4" t="n"/>
-    </row>
-    <row r="127" ht="26" customHeight="1">
-      <c r="A127" s="3" t="n">
-        <v>46253</v>
-      </c>
-      <c r="B127" s="4" t="inlineStr">
-        <is>
-          <t>Mercredi</t>
-        </is>
-      </c>
-      <c r="C127" s="12" t="inlineStr">
-        <is>
-          <t>Vélo</t>
-        </is>
-      </c>
-      <c r="D127" s="6" t="inlineStr">
-        <is>
-          <t>Sortie Z2 + SS — 125'</t>
-        </is>
-      </c>
-      <c r="E127" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="F127" s="6" t="inlineStr">
-        <is>
-          <t>Z2-Z3</t>
-        </is>
-      </c>
-      <c r="G127" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H127" s="7" t="inlineStr">
-        <is>
-          <t>20' EF | 2x24' SS @ 84% FTP — r=7' | Z2 reste | 15' RC
-NUTRITION : 48g/h</t>
-        </is>
-      </c>
-      <c r="I127" s="4" t="n"/>
-      <c r="J127" s="4" t="n">
-        <v>61</v>
-      </c>
-      <c r="K127" s="4" t="n"/>
-    </row>
-    <row r="128" ht="18" customHeight="1">
-      <c r="A128" s="3" t="n">
-        <v>46254</v>
-      </c>
-      <c r="B128" s="4" t="inlineStr">
-        <is>
-          <t>Jeudi</t>
-        </is>
-      </c>
-      <c r="C128" s="11" t="inlineStr">
-        <is>
-          <t>Course</t>
-        </is>
-      </c>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>EF — 30'</t>
-        </is>
-      </c>
-      <c r="E128" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>Z2</t>
-        </is>
-      </c>
-      <c r="G128" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H128" s="7" t="inlineStr">
-        <is>
-          <t>30' EF Z2 — économiser pour Luxembourg vélo</t>
-        </is>
-      </c>
-      <c r="I128" s="4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="J128" s="4" t="n"/>
-      <c r="K128" s="4" t="n"/>
+      <c r="L126" s="4" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="127" ht="15" customHeight="1">
+      <c r="A127" s="9" t="n"/>
+      <c r="B127" s="9" t="n"/>
+      <c r="C127" s="9" t="n"/>
+      <c r="D127" s="9" t="n"/>
+      <c r="E127" s="9" t="n"/>
+      <c r="F127" s="9" t="n"/>
+      <c r="G127" s="9" t="n"/>
+      <c r="H127" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PÉRIODE</t>
+        </is>
+      </c>
+      <c r="I127" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J127" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="K127" s="9" t="n"/>
+      <c r="L127" s="9" t="n"/>
+    </row>
+    <row r="128" ht="20" customHeight="1">
+      <c r="A128" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  21/08 → 24/08/2026   |   🚴 Luxembourg En Vélo — Camp vélo</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="39" customHeight="1">
       <c r="A129" s="3" t="n">
@@ -5286,7 +5636,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C129" s="12" t="inlineStr">
+      <c r="C129" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5319,6 +5669,9 @@
         <v>45</v>
       </c>
       <c r="K129" s="4" t="n"/>
+      <c r="L129" s="4" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="130" ht="39" customHeight="1">
       <c r="A130" s="3" t="n">
@@ -5329,7 +5682,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C130" s="12" t="inlineStr">
+      <c r="C130" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5362,6 +5715,9 @@
         <v>75</v>
       </c>
       <c r="K130" s="4" t="n"/>
+      <c r="L130" s="4" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="131" ht="26" customHeight="1">
       <c r="A131" s="3" t="n">
@@ -5372,7 +5728,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C131" s="12" t="inlineStr">
+      <c r="C131" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5404,76 +5760,79 @@
         <v>57</v>
       </c>
       <c r="K131" s="4" t="n"/>
-    </row>
-    <row r="132" ht="15" customHeight="1">
-      <c r="A132" s="9" t="n"/>
-      <c r="B132" s="9" t="n"/>
-      <c r="C132" s="9" t="n"/>
-      <c r="D132" s="9" t="n"/>
-      <c r="E132" s="9" t="n"/>
-      <c r="F132" s="9" t="n"/>
-      <c r="G132" s="9" t="n"/>
-      <c r="H132" s="10" t="inlineStr">
-        <is>
-          <t>Total semaine</t>
-        </is>
-      </c>
-      <c r="I132" s="9" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="J132" s="9" t="n">
-        <v>257</v>
-      </c>
-      <c r="K132" s="9" t="n"/>
-    </row>
-    <row r="133" ht="18" customHeight="1">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>Semaine 13 — 24/08 au 30/08/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="26" customHeight="1">
-      <c r="A134" s="3" t="n">
+      <c r="L131" s="4" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="132" ht="26" customHeight="1">
+      <c r="A132" s="3" t="n">
         <v>46258</v>
       </c>
-      <c r="B134" s="4" t="inlineStr">
+      <c r="B132" s="4" t="inlineStr">
         <is>
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C134" s="5" t="inlineStr">
+      <c r="C132" s="5" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="D134" s="6" t="inlineStr">
+      <c r="D132" s="6" t="inlineStr">
         <is>
           <t>OFF / Repos</t>
         </is>
       </c>
-      <c r="E134" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F134" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G134" s="4" t="n">
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F132" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H134" s="7" t="inlineStr">
+      <c r="H132" s="7" t="inlineStr">
         <is>
           <t>Retour Luxembourg En Vélo — repos
 Dernier grand repos avant semaine finale</t>
         </is>
       </c>
-      <c r="I134" s="4" t="n"/>
-      <c r="J134" s="4" t="n"/>
-      <c r="K134" s="4" t="n"/>
+      <c r="I132" s="4" t="n"/>
+      <c r="J132" s="4" t="n"/>
+      <c r="K132" s="4" t="n"/>
+      <c r="L132" s="4" t="n"/>
+    </row>
+    <row r="133" ht="15" customHeight="1">
+      <c r="A133" s="9" t="n"/>
+      <c r="B133" s="9" t="n"/>
+      <c r="C133" s="9" t="n"/>
+      <c r="D133" s="9" t="n"/>
+      <c r="E133" s="9" t="n"/>
+      <c r="F133" s="9" t="n"/>
+      <c r="G133" s="9" t="n"/>
+      <c r="H133" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL PÉRIODE</t>
+        </is>
+      </c>
+      <c r="I133" s="9" t="n"/>
+      <c r="J133" s="9" t="n">
+        <v>177</v>
+      </c>
+      <c r="K133" s="9" t="n"/>
+      <c r="L133" s="9" t="n"/>
+    </row>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  25/08 → 30/08/2026   |   Dernière semaine pré-plan IM | Nat WE 29-30 août</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="26" customHeight="1">
       <c r="A135" s="3" t="n">
@@ -5484,7 +5843,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C135" s="11" t="inlineStr">
+      <c r="C135" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -5508,7 +5867,7 @@
       <c r="H135" s="7" t="inlineStr">
         <is>
           <t>12' EF | 15' Z3 (148-154 bpm) | 15' Z2 | 6' RC
-Activation fraîche post-Luxembourg</t>
+Activation fraîche post-Luxembourg — terrain plat</t>
         </is>
       </c>
       <c r="I135" s="4" t="n">
@@ -5516,6 +5875,9 @@
       </c>
       <c r="J135" s="4" t="n"/>
       <c r="K135" s="4" t="n"/>
+      <c r="L135" s="4" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="n">
@@ -5526,7 +5888,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C136" s="12" t="inlineStr">
+      <c r="C136" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5557,6 +5919,9 @@
         <v>19</v>
       </c>
       <c r="K136" s="4" t="n"/>
+      <c r="L136" s="4" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="137" ht="26" customHeight="1">
       <c r="A137" s="3" t="n">
@@ -5567,7 +5932,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C137" s="12" t="inlineStr">
+      <c r="C137" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5599,6 +5964,9 @@
         <v>46</v>
       </c>
       <c r="K137" s="4" t="n"/>
+      <c r="L137" s="4" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="n">
@@ -5609,14 +5977,14 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C138" s="11" t="inlineStr">
+      <c r="C138" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>EF — 30'</t>
+          <t>EF — 30' plat</t>
         </is>
       </c>
       <c r="E138" s="4" t="n">
@@ -5632,7 +6000,7 @@
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile</t>
+          <t>30' EF Z2 facile — terrain plat</t>
         </is>
       </c>
       <c r="I138" s="4" t="n">
@@ -5640,6 +6008,9 @@
       </c>
       <c r="J138" s="4" t="n"/>
       <c r="K138" s="4" t="n"/>
+      <c r="L138" s="4" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="139" ht="39" customHeight="1">
       <c r="A139" s="3" t="n">
@@ -5650,7 +6021,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C139" s="11" t="inlineStr">
+      <c r="C139" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -5683,8 +6054,11 @@
       </c>
       <c r="J139" s="4" t="n"/>
       <c r="K139" s="4" t="n"/>
-    </row>
-    <row r="140" ht="39" customHeight="1">
+      <c r="L139" s="4" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="140" ht="26" customHeight="1">
       <c r="A140" s="3" t="n">
         <v>46263</v>
       </c>
@@ -5693,7 +6067,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C140" s="12" t="inlineStr">
+      <c r="C140" s="16" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5717,8 +6091,7 @@
       <c r="H140" s="7" t="inlineStr">
         <is>
           <t>118' Z2 (127-138 bpm) | 2x16' Z3 léger inclus
-NUTRITION : 46g/h
-Lundi : plan Ironman !</t>
+NUTRITION : 46g/h — Lundi : plan Ironman !</t>
         </is>
       </c>
       <c r="I140" s="4" t="n"/>
@@ -5726,8 +6099,11 @@
         <v>57</v>
       </c>
       <c r="K140" s="4" t="n"/>
-    </row>
-    <row r="141" ht="26" customHeight="1">
+      <c r="L140" s="4" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="n">
         <v>46263</v>
       </c>
@@ -5759,8 +6135,7 @@
       </c>
       <c r="H141" s="7" t="inlineStr">
         <is>
-          <t>4x50 facile | 10x50 éducatifs | 3x300 continu | 300 retour — 1 800 m
-Dernière nat avant plan IM</t>
+          <t>4x50 facile | 10x50 éducatifs | 3x300 continu | 300 retour — 1 800 m</t>
         </is>
       </c>
       <c r="I141" s="4" t="n"/>
@@ -5768,8 +6143,9 @@
       <c r="K141" s="4" t="n">
         <v>1800</v>
       </c>
-    </row>
-    <row r="142" ht="26" customHeight="1">
+      <c r="L141" s="4" t="n"/>
+    </row>
+    <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="n">
         <v>46264</v>
       </c>
@@ -5801,8 +6177,7 @@
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>200 EF | 2x700 continu (r=25'') | 200 retour — 1 800 m
-Bonne base aquatique construite !</t>
+          <t>200 EF | 2x700 continu (r=25'') | 200 retour — 1 800 m</t>
         </is>
       </c>
       <c r="I142" s="4" t="n"/>
@@ -5810,6 +6185,7 @@
       <c r="K142" s="4" t="n">
         <v>1800</v>
       </c>
+      <c r="L142" s="4" t="n"/>
     </row>
     <row r="143" ht="39" customHeight="1">
       <c r="A143" s="3" t="n">
@@ -5820,7 +6196,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C143" s="11" t="inlineStr">
+      <c r="C143" s="12" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -5853,6 +6229,9 @@
       </c>
       <c r="J143" s="4" t="n"/>
       <c r="K143" s="4" t="n"/>
+      <c r="L143" s="4" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1">
       <c r="A144" s="9" t="n"/>
@@ -5864,7 +6243,7 @@
       <c r="G144" s="9" t="n"/>
       <c r="H144" s="10" t="inlineStr">
         <is>
-          <t>Total semaine</t>
+          <t>TOTAL PÉRIODE</t>
         </is>
       </c>
       <c r="I144" s="9" t="n">
@@ -5876,22 +6255,40 @@
       <c r="K144" s="9" t="n">
         <v>3600</v>
       </c>
+      <c r="L144" s="9" t="n"/>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="21" t="inlineStr">
+        <is>
+          <t>TOTAL PRÉPARATION — 3 juin → 30 août 2026</t>
+        </is>
+      </c>
+      <c r="I145" s="22" t="n">
+        <v>274</v>
+      </c>
+      <c r="J145" s="22" t="n">
+        <v>1077</v>
+      </c>
+      <c r="K145" s="22" t="n">
+        <v>25300</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A56:K56"/>
-    <mergeCell ref="A69:K69"/>
-    <mergeCell ref="A92:K92"/>
-    <mergeCell ref="A101:K101"/>
-    <mergeCell ref="A82:K82"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="A110:K110"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A28:K28"/>
-    <mergeCell ref="A133:K133"/>
-    <mergeCell ref="A123:K123"/>
-    <mergeCell ref="A9:K9"/>
+  <mergeCells count="14">
+    <mergeCell ref="A145:H145"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A82:L82"/>
+    <mergeCell ref="A134:L134"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A128:L128"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A108:L108"/>
+    <mergeCell ref="A121:L121"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="A88:L88"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A56:L56"/>
+    <mergeCell ref="A69:L69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto sync 2026-06-12 05:55:02
</commit_message>
<xml_diff>
--- a/Marathon_programme.xlsx
+++ b/Marathon_programme.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preparation IM Final V2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Préparation IM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,24 +42,15 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <i val="1"/>
-      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -72,7 +64,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00795548"/>
+        <fgColor rgb="0037474F"/>
       </patternFill>
     </fill>
     <fill>
@@ -92,52 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001565C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFCCBC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E65100"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00880E4F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004A148C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00BBDEFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0037474F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000277BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B71C1C"/>
       </patternFill>
     </fill>
   </fills>
@@ -167,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -175,7 +127,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,43 +148,13 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -600,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -614,7 +536,6 @@
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -673,16 +594,11 @@
           <t>Distance (m) - Natation</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>D+</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  03/06 → 07/06/2026   |   Récupération totale — Pas de vélo, pas de CAP | Nat WE</t>
+          <t>Semaine 1 — 01/06 au 07/06/2026</t>
         </is>
       </c>
     </row>
@@ -729,7 +645,6 @@
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -772,7 +687,6 @@
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -814,7 +728,6 @@
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -859,7 +772,6 @@
       <c r="K6" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7" ht="39" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -903,7 +815,6 @@
       <c r="K7" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="L7" s="4" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="9" t="n"/>
@@ -915,7 +826,7 @@
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I8" s="9" t="n"/>
@@ -923,12 +834,11 @@
       <c r="K8" s="9" t="n">
         <v>2000</v>
       </c>
-      <c r="L8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  08/06 → 14/06/2026   |   Retour CAP très progressif PLAT STRICT — Pas de vélo | Nat WE</t>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 2 — 08/06 au 14/06/2026</t>
         </is>
       </c>
     </row>
@@ -972,7 +882,6 @@
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
-      <c r="L10" s="4" t="n"/>
     </row>
     <row r="11" ht="104" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -983,7 +892,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1021,9 +930,6 @@
       </c>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
-      <c r="L11" s="4" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="12" ht="39" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1067,7 +973,6 @@
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
     </row>
     <row r="13" ht="91" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1078,7 +983,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1115,9 +1020,6 @@
       </c>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -1159,7 +1061,6 @@
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1202,7 +1103,6 @@
       <c r="K15" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="L15" s="4" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1245,7 +1145,6 @@
       <c r="K16" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="L16" s="4" t="n"/>
     </row>
     <row r="17" ht="39" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1256,7 +1155,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1289,9 +1188,6 @@
       </c>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
-      <c r="L17" s="4" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="9" t="n"/>
@@ -1303,7 +1199,7 @@
       <c r="G18" s="9" t="n"/>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I18" s="9" t="n">
@@ -1313,12 +1209,11 @@
       <c r="K18" s="9" t="n">
         <v>2400</v>
       </c>
-      <c r="L18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  15/06 → 21/06/2026   |   Reprise CAP douce PLAT — Pas de vélo | Décision Malaga 20/06</t>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 3 — 15/06 au 21/06/2026</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1257,6 @@
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
     </row>
     <row r="21" ht="65" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1373,7 +1267,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1408,9 +1302,6 @@
       </c>
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="n"/>
-      <c r="L21" s="4" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -1452,7 +1343,6 @@
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="n"/>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -1463,7 +1353,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1497,9 +1387,6 @@
       </c>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -1541,7 +1428,6 @@
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
-      <c r="L24" s="4" t="n"/>
     </row>
     <row r="25" ht="108" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -1591,7 +1477,6 @@
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
-      <c r="L25" s="4" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="3" t="n">
@@ -1634,7 +1519,6 @@
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="9" t="n"/>
@@ -1646,7 +1530,7 @@
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I27" s="9" t="n">
@@ -1654,12 +1538,11 @@
       </c>
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
-      <c r="L27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  22/06 → 28/06/2026   |   🏔️ CAMP MALAGA — Montées CAP (DESCENTES À PIED) + Nat mer</t>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 4 — 22/06 au 28/06/2026</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1555,7 @@
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1710,9 +1593,6 @@
       </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="n">
-        <v>600</v>
-      </c>
     </row>
     <row r="30" ht="39" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -1756,7 +1636,6 @@
       <c r="K30" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="L30" s="4" t="n"/>
     </row>
     <row r="31" ht="78" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -1767,7 +1646,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1803,9 +1682,6 @@
       </c>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
-      <c r="L31" s="4" t="n">
-        <v>800</v>
-      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="3" t="n">
@@ -1847,7 +1723,6 @@
       <c r="K32" s="4" t="n">
         <v>750</v>
       </c>
-      <c r="L32" s="4" t="n"/>
     </row>
     <row r="33" ht="78" customHeight="1">
       <c r="A33" s="3" t="n">
@@ -1858,7 +1733,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -1894,9 +1769,6 @@
       </c>
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="n"/>
-      <c r="L33" s="4" t="n">
-        <v>1000</v>
-      </c>
     </row>
     <row r="34" ht="39" customHeight="1">
       <c r="A34" s="3" t="n">
@@ -1940,7 +1812,6 @@
       <c r="K34" s="4" t="n">
         <v>800</v>
       </c>
-      <c r="L34" s="4" t="n"/>
     </row>
     <row r="35" ht="39" customHeight="1">
       <c r="A35" s="3" t="n">
@@ -1984,7 +1855,6 @@
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -2027,7 +1897,6 @@
       <c r="K36" s="4" t="n">
         <v>550</v>
       </c>
-      <c r="L36" s="4" t="n"/>
     </row>
     <row r="37" ht="78" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -2038,7 +1907,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2074,9 +1943,6 @@
       </c>
       <c r="J37" s="4" t="n"/>
       <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="n">
-        <v>800</v>
-      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="3" t="n">
@@ -2118,7 +1984,6 @@
       <c r="K38" s="4" t="n">
         <v>800</v>
       </c>
-      <c r="L38" s="4" t="n"/>
     </row>
     <row r="39" ht="65" customHeight="1">
       <c r="A39" s="3" t="n">
@@ -2129,7 +1994,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2164,9 +2029,6 @@
       </c>
       <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="n">
-        <v>600</v>
-      </c>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -2209,7 +2071,6 @@
       <c r="K40" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="L40" s="4" t="n"/>
     </row>
     <row r="41" ht="39" customHeight="1">
       <c r="A41" s="3" t="n">
@@ -2253,7 +2114,6 @@
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="4" t="n"/>
       <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="9" t="n"/>
@@ -2265,7 +2125,7 @@
       <c r="G42" s="9" t="n"/>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I42" s="9" t="n">
@@ -2275,12 +2135,11 @@
       <c r="K42" s="9" t="n">
         <v>4100</v>
       </c>
-      <c r="L42" s="9" t="n"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  29/06 → 05/07/2026   |   Retour vélo 30/06 (cadence haute) + CAP plat + Nat WE</t>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 5 — 29/06 au 05/07/2026</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2183,6 @@
       <c r="I44" s="4" t="n"/>
       <c r="J44" s="4" t="n"/>
       <c r="K44" s="4" t="n"/>
-      <c r="L44" s="4" t="n"/>
     </row>
     <row r="45" ht="104" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -2335,7 +2193,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2373,9 +2231,6 @@
         <v>25</v>
       </c>
       <c r="K45" s="4" t="n"/>
-      <c r="L45" s="4" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="3" t="n">
@@ -2386,7 +2241,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2418,9 +2273,6 @@
       </c>
       <c r="J46" s="4" t="n"/>
       <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="47" ht="39" customHeight="1">
       <c r="A47" s="3" t="n">
@@ -2431,7 +2283,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C47" s="16" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2464,9 +2316,6 @@
         <v>39</v>
       </c>
       <c r="K47" s="4" t="n"/>
-      <c r="L47" s="4" t="n">
-        <v>105</v>
-      </c>
     </row>
     <row r="48" ht="52" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -2477,7 +2326,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2511,9 +2360,6 @@
         <v>26</v>
       </c>
       <c r="K48" s="4" t="n"/>
-      <c r="L48" s="4" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="3" t="n">
@@ -2524,7 +2370,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C49" s="12" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2555,9 +2401,6 @@
       </c>
       <c r="J49" s="4" t="n"/>
       <c r="K49" s="4" t="n"/>
-      <c r="L49" s="4" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="A50" s="3" t="n">
@@ -2568,7 +2411,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C50" s="12" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2600,9 +2443,6 @@
       </c>
       <c r="J50" s="4" t="n"/>
       <c r="K50" s="4" t="n"/>
-      <c r="L50" s="4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="51" ht="39" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -2613,7 +2453,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C51" s="16" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2646,9 +2486,6 @@
         <v>49</v>
       </c>
       <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="n">
-        <v>130</v>
-      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="3" t="n">
@@ -2690,7 +2527,6 @@
       <c r="K52" s="4" t="n">
         <v>1500</v>
       </c>
-      <c r="L52" s="4" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="3" t="n">
@@ -2732,7 +2568,6 @@
       <c r="K53" s="4" t="n">
         <v>1500</v>
       </c>
-      <c r="L53" s="4" t="n"/>
     </row>
     <row r="54" ht="52" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -2743,7 +2578,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr">
+      <c r="C54" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2777,9 +2612,6 @@
       </c>
       <c r="J54" s="4" t="n"/>
       <c r="K54" s="4" t="n"/>
-      <c r="L54" s="4" t="n">
-        <v>53</v>
-      </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="9" t="n"/>
@@ -2791,7 +2623,7 @@
       <c r="G55" s="9" t="n"/>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I55" s="9" t="n">
@@ -2803,12 +2635,11 @@
       <c r="K55" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="L55" s="9" t="n"/>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  06/07 → 12/07/2026   |   Build — Vélo + CAP + Nat WE 11-12 juil</t>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 6 — 06/07 au 12/07/2026</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2683,6 @@
       <c r="I57" s="4" t="n"/>
       <c r="J57" s="4" t="n"/>
       <c r="K57" s="4" t="n"/>
-      <c r="L57" s="4" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="3" t="n">
@@ -2863,7 +2693,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C58" s="16" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2894,9 +2724,6 @@
         <v>19</v>
       </c>
       <c r="K58" s="4" t="n"/>
-      <c r="L58" s="4" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="59" ht="52" customHeight="1">
       <c r="A59" s="3" t="n">
@@ -2907,7 +2734,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C59" s="12" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -2941,9 +2768,6 @@
       </c>
       <c r="J59" s="4" t="n"/>
       <c r="K59" s="4" t="n"/>
-      <c r="L59" s="4" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="60" ht="26" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -2954,7 +2778,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C60" s="16" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -2986,9 +2810,6 @@
         <v>44</v>
       </c>
       <c r="K60" s="4" t="n"/>
-      <c r="L60" s="4" t="n">
-        <v>117</v>
-      </c>
     </row>
     <row r="61" ht="78" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -2999,7 +2820,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C61" s="16" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3035,9 +2856,6 @@
         <v>31</v>
       </c>
       <c r="K61" s="4" t="n"/>
-      <c r="L61" s="4" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="3" t="n">
@@ -3048,7 +2866,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr">
+      <c r="C62" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3079,9 +2897,6 @@
       </c>
       <c r="J62" s="4" t="n"/>
       <c r="K62" s="4" t="n"/>
-      <c r="L62" s="4" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="3" t="n">
@@ -3092,7 +2907,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C63" s="12" t="inlineStr">
+      <c r="C63" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3124,9 +2939,6 @@
       </c>
       <c r="J63" s="4" t="n"/>
       <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="n">
-        <v>52</v>
-      </c>
     </row>
     <row r="64" ht="26" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -3137,7 +2949,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C64" s="16" t="inlineStr">
+      <c r="C64" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3169,9 +2981,6 @@
         <v>59</v>
       </c>
       <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n">
-        <v>157</v>
-      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="3" t="n">
@@ -3213,7 +3022,6 @@
       <c r="K65" s="4" t="n">
         <v>1700</v>
       </c>
-      <c r="L65" s="4" t="n"/>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="3" t="n">
@@ -3255,7 +3063,6 @@
       <c r="K66" s="4" t="n">
         <v>1700</v>
       </c>
-      <c r="L66" s="4" t="n"/>
     </row>
     <row r="67" ht="39" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -3266,7 +3073,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C67" s="12" t="inlineStr">
+      <c r="C67" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3299,9 +3106,6 @@
       </c>
       <c r="J67" s="4" t="n"/>
       <c r="K67" s="4" t="n"/>
-      <c r="L67" s="4" t="n">
-        <v>64</v>
-      </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="9" t="n"/>
@@ -3313,7 +3117,7 @@
       <c r="G68" s="9" t="n"/>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I68" s="9" t="n">
@@ -3325,12 +3129,11 @@
       <c r="K68" s="9" t="n">
         <v>3400</v>
       </c>
-      <c r="L68" s="9" t="n"/>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13/07 → 19/07/2026   |   Build pic pré-vacances — Vélo + CAP + Nat WE 18-19</t>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 7 — 13/07 au 19/07/2026</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3177,6 @@
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="4" t="n"/>
       <c r="K70" s="4" t="n"/>
-      <c r="L70" s="4" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="3" t="n">
@@ -3385,7 +3187,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C71" s="16" t="inlineStr">
+      <c r="C71" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3416,9 +3218,6 @@
         <v>19</v>
       </c>
       <c r="K71" s="4" t="n"/>
-      <c r="L71" s="4" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="72" ht="91" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -3429,7 +3228,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C72" s="12" t="inlineStr">
+      <c r="C72" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3466,9 +3265,6 @@
       </c>
       <c r="J72" s="4" t="n"/>
       <c r="K72" s="4" t="n"/>
-      <c r="L72" s="4" t="n">
-        <v>62</v>
-      </c>
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -3479,7 +3275,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C73" s="16" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3511,9 +3307,6 @@
         <v>51</v>
       </c>
       <c r="K73" s="4" t="n"/>
-      <c r="L73" s="4" t="n">
-        <v>136</v>
-      </c>
     </row>
     <row r="74" ht="65" customHeight="1">
       <c r="A74" s="3" t="n">
@@ -3524,7 +3317,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C74" s="16" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3559,9 +3352,6 @@
         <v>33</v>
       </c>
       <c r="K74" s="4" t="n"/>
-      <c r="L74" s="4" t="n">
-        <v>112</v>
-      </c>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -3572,7 +3362,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C75" s="12" t="inlineStr">
+      <c r="C75" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3603,9 +3393,6 @@
       </c>
       <c r="J75" s="4" t="n"/>
       <c r="K75" s="4" t="n"/>
-      <c r="L75" s="4" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="76" ht="26" customHeight="1">
       <c r="A76" s="3" t="n">
@@ -3616,7 +3403,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C76" s="12" t="inlineStr">
+      <c r="C76" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3648,9 +3435,6 @@
       </c>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
-      <c r="L76" s="4" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="77" ht="39" customHeight="1">
       <c r="A77" s="3" t="n">
@@ -3661,7 +3445,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C77" s="16" t="inlineStr">
+      <c r="C77" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3694,9 +3478,6 @@
         <v>68</v>
       </c>
       <c r="K77" s="4" t="n"/>
-      <c r="L77" s="4" t="n">
-        <v>182</v>
-      </c>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -3738,7 +3519,6 @@
       <c r="K78" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="L78" s="4" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="3" t="n">
@@ -3780,7 +3560,6 @@
       <c r="K79" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="L79" s="4" t="n"/>
     </row>
     <row r="80" ht="39" customHeight="1">
       <c r="A80" s="3" t="n">
@@ -3791,7 +3570,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr">
+      <c r="C80" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3824,9 +3603,6 @@
       </c>
       <c r="J80" s="4" t="n"/>
       <c r="K80" s="4" t="n"/>
-      <c r="L80" s="4" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="9" t="n"/>
@@ -3838,7 +3614,7 @@
       <c r="G81" s="9" t="n"/>
       <c r="H81" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I81" s="9" t="n">
@@ -3850,12 +3626,11 @@
       <c r="K81" s="9" t="n">
         <v>3600</v>
       </c>
-      <c r="L81" s="9" t="n"/>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  20/07 → 22/07/2026   |   Transition — dernière semaine avant vacances</t>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 8 — 20/07 au 26/07/2026</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3674,6 @@
       <c r="I83" s="4" t="n"/>
       <c r="J83" s="4" t="n"/>
       <c r="K83" s="4" t="n"/>
-      <c r="L83" s="4" t="n"/>
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="3" t="n">
@@ -3910,7 +3684,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C84" s="16" t="inlineStr">
+      <c r="C84" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -3942,9 +3716,6 @@
         <v>29</v>
       </c>
       <c r="K84" s="4" t="n"/>
-      <c r="L84" s="4" t="n">
-        <v>80</v>
-      </c>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -3955,7 +3726,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr">
+      <c r="C85" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -3986,9 +3757,6 @@
       </c>
       <c r="J85" s="4" t="n"/>
       <c r="K85" s="4" t="n"/>
-      <c r="L85" s="4" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="3" t="n">
@@ -3999,7 +3767,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C86" s="16" t="inlineStr">
+      <c r="C86" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -4030,46 +3798,96 @@
         <v>32</v>
       </c>
       <c r="K86" s="4" t="n"/>
-      <c r="L86" s="4" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="87" ht="15" customHeight="1">
-      <c r="A87" s="9" t="n"/>
-      <c r="B87" s="9" t="n"/>
-      <c r="C87" s="9" t="n"/>
-      <c r="D87" s="9" t="n"/>
-      <c r="E87" s="9" t="n"/>
-      <c r="F87" s="9" t="n"/>
-      <c r="G87" s="9" t="n"/>
-      <c r="H87" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL PÉRIODE</t>
-        </is>
-      </c>
-      <c r="I87" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="J87" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="K87" s="9" t="n"/>
-      <c r="L87" s="9" t="n"/>
-    </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  23/07 → 09/08/2026   |   🇮🇹🇬🇷 VACANCES Italie + Grèce — ZÉRO SÉANCE</t>
-        </is>
-      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="3" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>🇮🇹 Voyage Luxembourg→Florence — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="n"/>
+      <c r="J87" s="4" t="n"/>
+      <c r="K87" s="4" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="3" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>🇮🇹 Florence (excursion Sienne) — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="3" t="n">
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Samedi</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -4097,21 +3915,20 @@
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>🇮🇹 Voyage Luxembourg→Florence — ZÉRO SÉANCE</t>
+          <t>🇮🇹 Florence — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I89" s="4" t="n"/>
       <c r="J89" s="4" t="n"/>
       <c r="K89" s="4" t="n"/>
-      <c r="L89" s="4" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="3" t="n">
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Vendredi</t>
+          <t>Dimanche</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -4139,97 +3956,40 @@
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>🇮🇹 Florence (excursion Sienne) — ZÉRO SÉANCE</t>
+          <t>🇮🇹 Florence→Rome — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I90" s="4" t="n"/>
       <c r="J90" s="4" t="n"/>
       <c r="K90" s="4" t="n"/>
-      <c r="L90" s="4" t="n"/>
-    </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="3" t="n">
-        <v>46228</v>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>Samedi</t>
-        </is>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F91" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G91" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H91" s="7" t="inlineStr">
-        <is>
-          <t>🇮🇹 Florence — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I91" s="4" t="n"/>
-      <c r="J91" s="4" t="n"/>
-      <c r="K91" s="4" t="n"/>
-      <c r="L91" s="4" t="n"/>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="9" t="n"/>
+      <c r="B91" s="9" t="n"/>
+      <c r="C91" s="9" t="n"/>
+      <c r="D91" s="9" t="n"/>
+      <c r="E91" s="9" t="n"/>
+      <c r="F91" s="9" t="n"/>
+      <c r="G91" s="9" t="n"/>
+      <c r="H91" s="10" t="inlineStr">
+        <is>
+          <t>Total semaine</t>
+        </is>
+      </c>
+      <c r="I91" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J91" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="K91" s="9" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="3" t="n">
-        <v>46229</v>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>Dimanche</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F92" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G92" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H92" s="7" t="inlineStr">
-        <is>
-          <t>🇮🇹 Florence→Rome — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I92" s="4" t="n"/>
-      <c r="J92" s="4" t="n"/>
-      <c r="K92" s="4" t="n"/>
-      <c r="L92" s="4" t="n"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 9 — 27/07 au 02/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="3" t="n">
@@ -4271,7 +4031,6 @@
       <c r="I93" s="4" t="n"/>
       <c r="J93" s="4" t="n"/>
       <c r="K93" s="4" t="n"/>
-      <c r="L93" s="4" t="n"/>
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="3" t="n">
@@ -4313,7 +4072,6 @@
       <c r="I94" s="4" t="n"/>
       <c r="J94" s="4" t="n"/>
       <c r="K94" s="4" t="n"/>
-      <c r="L94" s="4" t="n"/>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="3" t="n">
@@ -4355,7 +4113,6 @@
       <c r="I95" s="4" t="n"/>
       <c r="J95" s="4" t="n"/>
       <c r="K95" s="4" t="n"/>
-      <c r="L95" s="4" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="3" t="n">
@@ -4397,7 +4154,6 @@
       <c r="I96" s="4" t="n"/>
       <c r="J96" s="4" t="n"/>
       <c r="K96" s="4" t="n"/>
-      <c r="L96" s="4" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="3" t="n">
@@ -4439,7 +4195,6 @@
       <c r="I97" s="4" t="n"/>
       <c r="J97" s="4" t="n"/>
       <c r="K97" s="4" t="n"/>
-      <c r="L97" s="4" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="3" t="n">
@@ -4481,7 +4236,6 @@
       <c r="I98" s="4" t="n"/>
       <c r="J98" s="4" t="n"/>
       <c r="K98" s="4" t="n"/>
-      <c r="L98" s="4" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="3" t="n">
@@ -4523,99 +4277,38 @@
       <c r="I99" s="4" t="n"/>
       <c r="J99" s="4" t="n"/>
       <c r="K99" s="4" t="n"/>
-      <c r="L99" s="4" t="n"/>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="3" t="n">
-        <v>46237</v>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>Lundi</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D100" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E100" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F100" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G100" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H100" s="7" t="inlineStr">
-        <is>
-          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I100" s="4" t="n"/>
-      <c r="J100" s="4" t="n"/>
-      <c r="K100" s="4" t="n"/>
-      <c r="L100" s="4" t="n"/>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="9" t="n"/>
+      <c r="B100" s="9" t="n"/>
+      <c r="C100" s="9" t="n"/>
+      <c r="D100" s="9" t="n"/>
+      <c r="E100" s="9" t="n"/>
+      <c r="F100" s="9" t="n"/>
+      <c r="G100" s="9" t="n"/>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>Total semaine</t>
+        </is>
+      </c>
+      <c r="I100" s="9" t="n"/>
+      <c r="J100" s="9" t="n"/>
+      <c r="K100" s="9" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="3" t="n">
-        <v>46238</v>
-      </c>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D101" s="6" t="inlineStr">
-        <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E101" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G101" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H101" s="7" t="inlineStr">
-        <is>
-          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
-        </is>
-      </c>
-      <c r="I101" s="4" t="n"/>
-      <c r="J101" s="4" t="n"/>
-      <c r="K101" s="4" t="n"/>
-      <c r="L101" s="4" t="n"/>
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 10 — 03/08 au 09/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="3" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Mercredi</t>
+          <t>Lundi</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
@@ -4649,15 +4342,14 @@
       <c r="I102" s="4" t="n"/>
       <c r="J102" s="4" t="n"/>
       <c r="K102" s="4" t="n"/>
-      <c r="L102" s="4" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="3" t="n">
-        <v>46240</v>
+        <v>46238</v>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Jeudi</t>
+          <t>Mardi</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
@@ -4691,15 +4383,14 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
       <c r="K103" s="4" t="n"/>
-      <c r="L103" s="4" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="3" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Vendredi</t>
+          <t>Mercredi</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
@@ -4733,15 +4424,14 @@
       <c r="I104" s="4" t="n"/>
       <c r="J104" s="4" t="n"/>
       <c r="K104" s="4" t="n"/>
-      <c r="L104" s="4" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="3" t="n">
-        <v>46242</v>
+        <v>46240</v>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Samedi</t>
+          <t>Jeudi</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
@@ -4775,15 +4465,14 @@
       <c r="I105" s="4" t="n"/>
       <c r="J105" s="4" t="n"/>
       <c r="K105" s="4" t="n"/>
-      <c r="L105" s="4" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="3" t="n">
-        <v>46243</v>
+        <v>46241</v>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Dimanche</t>
+          <t>Vendredi</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
@@ -4811,72 +4500,152 @@
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>🇬🇷→🇱🇺 Retour Thessalonique→Luxembourg — ZÉRO SÉANCE</t>
+          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
         </is>
       </c>
       <c r="I106" s="4" t="n"/>
       <c r="J106" s="4" t="n"/>
       <c r="K106" s="4" t="n"/>
-      <c r="L106" s="4" t="n"/>
-    </row>
-    <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="9" t="n"/>
-      <c r="C107" s="9" t="n"/>
-      <c r="D107" s="9" t="n"/>
-      <c r="E107" s="9" t="n"/>
-      <c r="F107" s="9" t="n"/>
-      <c r="G107" s="9" t="n"/>
-      <c r="H107" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL PÉRIODE</t>
-        </is>
-      </c>
-      <c r="I107" s="9" t="n"/>
-      <c r="J107" s="9" t="n"/>
-      <c r="K107" s="9" t="n"/>
-      <c r="L107" s="9" t="n"/>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  10/08 → 16/08/2026   |   ⚡ REPRISE CRITIQUE J-21 plan IM | Nat WE 15-16 août</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="91" customHeight="1">
-      <c r="A109" s="3" t="n">
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="n"/>
+      <c r="J107" s="4" t="n"/>
+      <c r="K107" s="4" t="n"/>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H108" s="7" t="inlineStr">
+        <is>
+          <t>🇬🇷→🇱🇺 Retour Thessalonique→Luxembourg — ZÉRO SÉANCE</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="n"/>
+      <c r="J108" s="4" t="n"/>
+      <c r="K108" s="4" t="n"/>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="9" t="n"/>
+      <c r="B109" s="9" t="n"/>
+      <c r="C109" s="9" t="n"/>
+      <c r="D109" s="9" t="n"/>
+      <c r="E109" s="9" t="n"/>
+      <c r="F109" s="9" t="n"/>
+      <c r="G109" s="9" t="n"/>
+      <c r="H109" s="10" t="inlineStr">
+        <is>
+          <t>Total semaine</t>
+        </is>
+      </c>
+      <c r="I109" s="9" t="n"/>
+      <c r="J109" s="9" t="n"/>
+      <c r="K109" s="9" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 11 — 10/08 au 16/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="91" customHeight="1">
+      <c r="A111" s="3" t="n">
         <v>46244</v>
       </c>
-      <c r="B109" s="4" t="inlineStr">
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C109" s="5" t="inlineStr">
+      <c r="C111" s="5" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="D109" s="6" t="inlineStr">
+      <c r="D111" s="6" t="inlineStr">
         <is>
           <t>OFF / Repos</t>
         </is>
       </c>
-      <c r="E109" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G109" s="4" t="n">
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H109" s="7" t="inlineStr">
+      <c r="H111" s="7" t="inlineStr">
         <is>
           <t>Repos — récup voyage retour Grèce
 J-21 plan Ironman — reprise ultra-progressive
@@ -4886,42 +4655,41 @@
 Sem 3 (24-30) : Volume -20% — arriver FRAIS le 31 août</t>
         </is>
       </c>
-      <c r="I109" s="4" t="n"/>
-      <c r="J109" s="4" t="n"/>
-      <c r="K109" s="4" t="n"/>
-      <c r="L109" s="4" t="n"/>
-    </row>
-    <row r="110" ht="52" customHeight="1">
-      <c r="A110" s="3" t="n">
+      <c r="I111" s="4" t="n"/>
+      <c r="J111" s="4" t="n"/>
+      <c r="K111" s="4" t="n"/>
+    </row>
+    <row r="112" ht="52" customHeight="1">
+      <c r="A112" s="3" t="n">
         <v>46245</v>
       </c>
-      <c r="B110" s="4" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C110" s="12" t="inlineStr">
+      <c r="C112" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
+      <c r="D112" s="6" t="inlineStr">
         <is>
           <t>EF reprise — post-vacances plat</t>
         </is>
       </c>
-      <c r="E110" s="4" t="n">
+      <c r="E112" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="F110" s="6" t="inlineStr">
+      <c r="F112" s="6" t="inlineStr">
         <is>
           <t>Z1-Z2</t>
         </is>
       </c>
-      <c r="G110" s="4" t="n">
+      <c r="G112" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H110" s="7" t="inlineStr">
+      <c r="H112" s="7" t="inlineStr">
         <is>
           <t>35' EF Z2 (120-133 bpm) — reprise très douce
 18 jours sans séance — ne pas forcer
@@ -4929,182 +4697,170 @@
 Marche-course si besoin</t>
         </is>
       </c>
-      <c r="I110" s="4" t="n">
+      <c r="I112" s="4" t="n">
         <v>6.5</v>
       </c>
-      <c r="J110" s="4" t="n"/>
-      <c r="K110" s="4" t="n"/>
-      <c r="L110" s="4" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="111" ht="39" customHeight="1">
-      <c r="A111" s="3" t="n">
+      <c r="J112" s="4" t="n"/>
+      <c r="K112" s="4" t="n"/>
+    </row>
+    <row r="113" ht="39" customHeight="1">
+      <c r="A113" s="3" t="n">
         <v>46245</v>
       </c>
-      <c r="B111" s="4" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C111" s="16" t="inlineStr">
+      <c r="C113" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D111" s="6" t="inlineStr">
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>Vélo reprise Z2 — 48' (cadence haute)</t>
         </is>
       </c>
-      <c r="E111" s="4" t="n">
+      <c r="E113" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="F111" s="6" t="inlineStr">
+      <c r="F113" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G111" s="4" t="n">
+      <c r="G113" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H111" s="7" t="inlineStr">
+      <c r="H113" s="7" t="inlineStr">
         <is>
           <t>48' Z2 — reprendre les jambes vélo
 Cadence 90-95 rpm — jamais &gt; Z2
 Genou : cadence haute encore obligatoire</t>
         </is>
       </c>
-      <c r="I111" s="4" t="n"/>
-      <c r="J111" s="4" t="n">
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="K111" s="4" t="n"/>
-      <c r="L111" s="4" t="n">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="112" ht="39" customHeight="1">
-      <c r="A112" s="3" t="n">
+      <c r="K113" s="4" t="n"/>
+    </row>
+    <row r="114" ht="39" customHeight="1">
+      <c r="A114" s="3" t="n">
         <v>46246</v>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C112" s="16" t="inlineStr">
+      <c r="C114" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>Sortie Z2 + SS reprise — 115'</t>
         </is>
       </c>
-      <c r="E112" s="4" t="n">
+      <c r="E114" s="4" t="n">
         <v>115</v>
       </c>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="F114" s="6" t="inlineStr">
         <is>
           <t>Z2-Z3</t>
         </is>
       </c>
-      <c r="G112" s="4" t="n">
+      <c r="G114" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H112" s="7" t="inlineStr">
+      <c r="H114" s="7" t="inlineStr">
         <is>
           <t>20' EF | 2x20' SS @ 81% FTP — r=6' | Z2 reste | 15' RC
 Reprise progressive — intensité réduite
 NUTRITION : 43g/h</t>
         </is>
       </c>
-      <c r="I112" s="4" t="n"/>
-      <c r="J112" s="4" t="n">
+      <c r="I114" s="4" t="n"/>
+      <c r="J114" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="K112" s="4" t="n"/>
-      <c r="L112" s="4" t="n">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="3" t="n">
+      <c r="K114" s="4" t="n"/>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="3" t="n">
         <v>46247</v>
       </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C113" s="12" t="inlineStr">
+      <c r="C115" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D113" s="6" t="inlineStr">
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>EF — 33' plat</t>
         </is>
       </c>
-      <c r="E113" s="4" t="n">
+      <c r="E115" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="F113" s="6" t="inlineStr">
+      <c r="F115" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G113" s="4" t="n">
+      <c r="G115" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H113" s="7" t="inlineStr">
+      <c r="H115" s="7" t="inlineStr">
         <is>
           <t>33' EF Z2 facile — terrain plat</t>
         </is>
       </c>
-      <c r="I113" s="4" t="n">
+      <c r="I115" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J113" s="4" t="n"/>
-      <c r="K113" s="4" t="n"/>
-      <c r="L113" s="4" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="114" ht="52" customHeight="1">
-      <c r="A114" s="3" t="n">
+      <c r="J115" s="4" t="n"/>
+      <c r="K115" s="4" t="n"/>
+    </row>
+    <row r="116" ht="52" customHeight="1">
+      <c r="A116" s="3" t="n">
         <v>46248</v>
       </c>
-      <c r="B114" s="4" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C114" s="16" t="inlineStr">
+      <c r="C116" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="D116" s="6" t="inlineStr">
         <is>
           <t>Force légère — 60' (si asymptomatique)</t>
         </is>
       </c>
-      <c r="E114" s="4" t="n">
+      <c r="E116" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="F114" s="6" t="inlineStr">
+      <c r="F116" s="6" t="inlineStr">
         <is>
           <t>Z2-Z3</t>
         </is>
       </c>
-      <c r="G114" s="4" t="n">
+      <c r="G116" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H114" s="7" t="inlineStr">
+      <c r="H116" s="7" t="inlineStr">
         <is>
           <t>10' EF
 SI genou asymptomatique :
@@ -5112,384 +4868,365 @@
 SINON : cadence haute 92-97 rpm uniquement</t>
         </is>
       </c>
-      <c r="I114" s="4" t="n"/>
-      <c r="J114" s="4" t="n">
+      <c r="I116" s="4" t="n"/>
+      <c r="J116" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="K114" s="4" t="n"/>
-      <c r="L114" s="4" t="n">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="115" ht="39" customHeight="1">
-      <c r="A115" s="3" t="n">
+      <c r="K116" s="4" t="n"/>
+    </row>
+    <row r="117" ht="39" customHeight="1">
+      <c r="A117" s="3" t="n">
         <v>46248</v>
       </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C115" s="12" t="inlineStr">
+      <c r="C117" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>Tempo très léger — 2x12'</t>
         </is>
       </c>
-      <c r="E115" s="4" t="n">
+      <c r="E117" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="F115" s="6" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>Z3</t>
         </is>
       </c>
-      <c r="G115" s="4" t="n">
+      <c r="G117" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H115" s="7" t="inlineStr">
+      <c r="H117" s="7" t="inlineStr">
         <is>
           <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
 Post-vacances — très contrôlé
 FC cible : 147-153 bpm max — terrain plat</t>
         </is>
       </c>
-      <c r="I115" s="4" t="n">
+      <c r="I117" s="4" t="n">
         <v>8.5</v>
       </c>
-      <c r="J115" s="4" t="n"/>
-      <c r="K115" s="4" t="n"/>
-      <c r="L115" s="4" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="116" ht="26" customHeight="1">
-      <c r="A116" s="3" t="n">
+      <c r="J117" s="4" t="n"/>
+      <c r="K117" s="4" t="n"/>
+    </row>
+    <row r="118" ht="26" customHeight="1">
+      <c r="A118" s="3" t="n">
         <v>46249</v>
       </c>
-      <c r="B116" s="4" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C116" s="16" t="inlineStr">
+      <c r="C118" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>Sortie longue Z2 — 140'</t>
         </is>
       </c>
-      <c r="E116" s="4" t="n">
+      <c r="E118" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="F118" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G116" s="4" t="n">
+      <c r="G118" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H116" s="7" t="inlineStr">
+      <c r="H118" s="7" t="inlineStr">
         <is>
           <t>140' Z2 (127-140 bpm) | 2x22' Z3 inclus — r=10'
 NUTRITION : 47g/h | Cadence 85-92 rpm</t>
         </is>
       </c>
-      <c r="I116" s="4" t="n"/>
-      <c r="J116" s="4" t="n">
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="K116" s="4" t="n"/>
-      <c r="L116" s="4" t="n">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="3" t="n">
+      <c r="K118" s="4" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="3" t="n">
         <v>46249</v>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C117" s="8" t="inlineStr">
+      <c r="C119" s="8" t="inlineStr">
         <is>
           <t>Natation</t>
         </is>
       </c>
-      <c r="D117" s="6" t="inlineStr">
+      <c r="D119" s="6" t="inlineStr">
         <is>
           <t>🏊 Natation technique — 1600m</t>
         </is>
       </c>
-      <c r="E117" s="4" t="n">
+      <c r="E119" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="F117" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G117" s="4" t="n">
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H117" s="7" t="inlineStr">
+      <c r="H119" s="7" t="inlineStr">
         <is>
           <t>4x50 facile | 10x50 éducatifs | 3x250 continu | 350 retour — 1 600 m</t>
         </is>
       </c>
-      <c r="I117" s="4" t="n"/>
-      <c r="J117" s="4" t="n"/>
-      <c r="K117" s="4" t="n">
+      <c r="I119" s="4" t="n"/>
+      <c r="J119" s="4" t="n"/>
+      <c r="K119" s="4" t="n">
         <v>1600</v>
       </c>
-      <c r="L117" s="4" t="n"/>
-    </row>
-    <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="3" t="n">
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="3" t="n">
         <v>46250</v>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C118" s="8" t="inlineStr">
+      <c r="C120" s="8" t="inlineStr">
         <is>
           <t>Natation</t>
         </is>
       </c>
-      <c r="D118" s="6" t="inlineStr">
+      <c r="D120" s="6" t="inlineStr">
         <is>
           <t>🏊 Natation endurance — 1600m</t>
         </is>
       </c>
-      <c r="E118" s="4" t="n">
+      <c r="E120" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="F118" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G118" s="4" t="n">
+      <c r="F120" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H118" s="7" t="inlineStr">
+      <c r="H120" s="7" t="inlineStr">
         <is>
           <t>200 EF | 2x600 continu (r=25'') | 200 retour — 1 600 m</t>
         </is>
       </c>
-      <c r="I118" s="4" t="n"/>
-      <c r="J118" s="4" t="n"/>
-      <c r="K118" s="4" t="n">
+      <c r="I120" s="4" t="n"/>
+      <c r="J120" s="4" t="n"/>
+      <c r="K120" s="4" t="n">
         <v>1600</v>
       </c>
-      <c r="L118" s="4" t="n"/>
-    </row>
-    <row r="119" ht="39" customHeight="1">
-      <c r="A119" s="3" t="n">
+    </row>
+    <row r="121" ht="39" customHeight="1">
+      <c r="A121" s="3" t="n">
         <v>46250</v>
       </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C119" s="12" t="inlineStr">
+      <c r="C121" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D119" s="6" t="inlineStr">
+      <c r="D121" s="6" t="inlineStr">
         <is>
           <t>Sortie longue Z2 — 78' (plat/vallonné)</t>
         </is>
       </c>
-      <c r="E119" s="4" t="n">
+      <c r="E121" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="F119" s="6" t="inlineStr">
+      <c r="F121" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G119" s="4" t="n">
+      <c r="G121" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H119" s="7" t="inlineStr">
+      <c r="H121" s="7" t="inlineStr">
         <is>
           <t>78' Z2 (127-140 bpm) — foncier solide
 Allure conversationnelle
 Genou : terrain plat ou légèrement vallonné</t>
         </is>
       </c>
-      <c r="I119" s="4" t="n">
+      <c r="I121" s="4" t="n">
         <v>14.5</v>
       </c>
-      <c r="J119" s="4" t="n"/>
-      <c r="K119" s="4" t="n"/>
-      <c r="L119" s="4" t="n">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="9" t="n"/>
-      <c r="B120" s="9" t="n"/>
-      <c r="C120" s="9" t="n"/>
-      <c r="D120" s="9" t="n"/>
-      <c r="E120" s="9" t="n"/>
-      <c r="F120" s="9" t="n"/>
-      <c r="G120" s="9" t="n"/>
-      <c r="H120" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL PÉRIODE</t>
-        </is>
-      </c>
-      <c r="I120" s="9" t="n">
+      <c r="J121" s="4" t="n"/>
+      <c r="K121" s="4" t="n"/>
+    </row>
+    <row r="122" ht="15" customHeight="1">
+      <c r="A122" s="9" t="n"/>
+      <c r="B122" s="9" t="n"/>
+      <c r="C122" s="9" t="n"/>
+      <c r="D122" s="9" t="n"/>
+      <c r="E122" s="9" t="n"/>
+      <c r="F122" s="9" t="n"/>
+      <c r="G122" s="9" t="n"/>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>Total semaine</t>
+        </is>
+      </c>
+      <c r="I122" s="9" t="n">
         <v>35.5</v>
       </c>
-      <c r="J120" s="9" t="n">
+      <c r="J122" s="9" t="n">
         <v>174</v>
       </c>
-      <c r="K120" s="9" t="n">
+      <c r="K122" s="9" t="n">
         <v>3200</v>
       </c>
-      <c r="L120" s="9" t="n"/>
-    </row>
-    <row r="121" ht="20" customHeight="1">
-      <c r="A121" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  17/08 → 20/08/2026   |   Build final 17-20 août</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="18" customHeight="1">
-      <c r="A122" s="3" t="n">
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 12 — 17/08 au 23/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="A124" s="3" t="n">
         <v>46251</v>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="D122" s="6" t="inlineStr">
+      <c r="D124" s="6" t="inlineStr">
         <is>
           <t>OFF / Repos</t>
         </is>
       </c>
-      <c r="E122" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G122" s="4" t="n">
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H122" s="7" t="inlineStr">
+      <c r="H124" s="7" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="I122" s="4" t="n"/>
-      <c r="J122" s="4" t="n"/>
-      <c r="K122" s="4" t="n"/>
-      <c r="L122" s="4" t="n"/>
-    </row>
-    <row r="123" ht="18" customHeight="1">
-      <c r="A123" s="3" t="n">
+      <c r="I124" s="4" t="n"/>
+      <c r="J124" s="4" t="n"/>
+      <c r="K124" s="4" t="n"/>
+    </row>
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="3" t="n">
         <v>46252</v>
       </c>
-      <c r="B123" s="4" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C123" s="16" t="inlineStr">
+      <c r="C125" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr">
+      <c r="D125" s="6" t="inlineStr">
         <is>
           <t>Vélo récup Z2 — 42'</t>
         </is>
       </c>
-      <c r="E123" s="4" t="n">
+      <c r="E125" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="F123" s="6" t="inlineStr">
+      <c r="F125" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G123" s="4" t="n">
+      <c r="G125" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H123" s="7" t="inlineStr">
+      <c r="H125" s="7" t="inlineStr">
         <is>
           <t>42' Z2 récup — cadence 90-95 rpm</t>
         </is>
       </c>
-      <c r="I123" s="4" t="n"/>
-      <c r="J123" s="4" t="n">
+      <c r="I125" s="4" t="n"/>
+      <c r="J125" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="K123" s="4" t="n"/>
-      <c r="L123" s="4" t="n">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="124" ht="91" customHeight="1">
-      <c r="A124" s="3" t="n">
+      <c r="K125" s="4" t="n"/>
+    </row>
+    <row r="126" ht="91" customHeight="1">
+      <c r="A126" s="3" t="n">
         <v>46252</v>
       </c>
-      <c r="B124" s="4" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C124" s="12" t="inlineStr">
+      <c r="C126" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D124" s="6" t="inlineStr">
+      <c r="D126" s="6" t="inlineStr">
         <is>
           <t>Qualité — 5x2000m progressif</t>
         </is>
       </c>
-      <c r="E124" s="4" t="n">
+      <c r="E126" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="F124" s="6" t="inlineStr">
+      <c r="F126" s="6" t="inlineStr">
         <is>
           <t>Z3-Z4</t>
         </is>
       </c>
-      <c r="G124" s="4" t="n">
+      <c r="G126" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H124" s="7" t="inlineStr">
+      <c r="H126" s="7" t="inlineStr">
         <is>
           <t>12' EF
 5x2000m progressif :
@@ -5500,132 +5237,94 @@
 10' RC — terrain plat</t>
         </is>
       </c>
-      <c r="I124" s="4" t="n">
+      <c r="I126" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="J124" s="4" t="n"/>
-      <c r="K124" s="4" t="n"/>
-      <c r="L124" s="4" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="125" ht="26" customHeight="1">
-      <c r="A125" s="3" t="n">
+      <c r="J126" s="4" t="n"/>
+      <c r="K126" s="4" t="n"/>
+    </row>
+    <row r="127" ht="26" customHeight="1">
+      <c r="A127" s="3" t="n">
         <v>46253</v>
       </c>
-      <c r="B125" s="4" t="inlineStr">
+      <c r="B127" s="4" t="inlineStr">
         <is>
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C125" s="16" t="inlineStr">
+      <c r="C127" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
       </c>
-      <c r="D125" s="6" t="inlineStr">
+      <c r="D127" s="6" t="inlineStr">
         <is>
           <t>Sortie Z2 + SS — 125'</t>
         </is>
       </c>
-      <c r="E125" s="4" t="n">
+      <c r="E127" s="4" t="n">
         <v>125</v>
       </c>
-      <c r="F125" s="6" t="inlineStr">
+      <c r="F127" s="6" t="inlineStr">
         <is>
           <t>Z2-Z3</t>
         </is>
       </c>
-      <c r="G125" s="4" t="n">
+      <c r="G127" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H125" s="7" t="inlineStr">
+      <c r="H127" s="7" t="inlineStr">
         <is>
           <t>20' EF | 2x24' SS @ 84% FTP — r=7' | Z2 reste | 15' RC
 NUTRITION : 48g/h</t>
         </is>
       </c>
-      <c r="I125" s="4" t="n"/>
-      <c r="J125" s="4" t="n">
+      <c r="I127" s="4" t="n"/>
+      <c r="J127" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="K125" s="4" t="n"/>
-      <c r="L125" s="4" t="n">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="126" ht="18" customHeight="1">
-      <c r="A126" s="3" t="n">
+      <c r="K127" s="4" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="3" t="n">
         <v>46254</v>
       </c>
-      <c r="B126" s="4" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C126" s="12" t="inlineStr">
+      <c r="C128" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D126" s="6" t="inlineStr">
+      <c r="D128" s="6" t="inlineStr">
         <is>
           <t>EF — 30'</t>
         </is>
       </c>
-      <c r="E126" s="4" t="n">
+      <c r="E128" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="F126" s="6" t="inlineStr">
+      <c r="F128" s="6" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G126" s="4" t="n">
+      <c r="G128" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H126" s="7" t="inlineStr">
+      <c r="H128" s="7" t="inlineStr">
         <is>
           <t>30' EF Z2 — économiser pour Luxembourg vélo</t>
         </is>
       </c>
-      <c r="I126" s="4" t="n">
+      <c r="I128" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="J126" s="4" t="n"/>
-      <c r="K126" s="4" t="n"/>
-      <c r="L126" s="4" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="127" ht="15" customHeight="1">
-      <c r="A127" s="9" t="n"/>
-      <c r="B127" s="9" t="n"/>
-      <c r="C127" s="9" t="n"/>
-      <c r="D127" s="9" t="n"/>
-      <c r="E127" s="9" t="n"/>
-      <c r="F127" s="9" t="n"/>
-      <c r="G127" s="9" t="n"/>
-      <c r="H127" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL PÉRIODE</t>
-        </is>
-      </c>
-      <c r="I127" s="9" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="J127" s="9" t="n">
-        <v>80</v>
-      </c>
-      <c r="K127" s="9" t="n"/>
-      <c r="L127" s="9" t="n"/>
-    </row>
-    <row r="128" ht="20" customHeight="1">
-      <c r="A128" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  21/08 → 24/08/2026   |   🚴 Luxembourg En Vélo — Camp vélo</t>
-        </is>
-      </c>
+      <c r="J128" s="4" t="n"/>
+      <c r="K128" s="4" t="n"/>
     </row>
     <row r="129" ht="39" customHeight="1">
       <c r="A129" s="3" t="n">
@@ -5636,7 +5335,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C129" s="16" t="inlineStr">
+      <c r="C129" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5669,9 +5368,6 @@
         <v>45</v>
       </c>
       <c r="K129" s="4" t="n"/>
-      <c r="L129" s="4" t="n">
-        <v>140</v>
-      </c>
     </row>
     <row r="130" ht="39" customHeight="1">
       <c r="A130" s="3" t="n">
@@ -5682,7 +5378,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C130" s="16" t="inlineStr">
+      <c r="C130" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5715,9 +5411,6 @@
         <v>75</v>
       </c>
       <c r="K130" s="4" t="n"/>
-      <c r="L130" s="4" t="n">
-        <v>240</v>
-      </c>
     </row>
     <row r="131" ht="26" customHeight="1">
       <c r="A131" s="3" t="n">
@@ -5728,7 +5421,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C131" s="16" t="inlineStr">
+      <c r="C131" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5760,79 +5453,76 @@
         <v>57</v>
       </c>
       <c r="K131" s="4" t="n"/>
-      <c r="L131" s="4" t="n">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="132" ht="26" customHeight="1">
-      <c r="A132" s="3" t="n">
+    </row>
+    <row r="132" ht="15" customHeight="1">
+      <c r="A132" s="9" t="n"/>
+      <c r="B132" s="9" t="n"/>
+      <c r="C132" s="9" t="n"/>
+      <c r="D132" s="9" t="n"/>
+      <c r="E132" s="9" t="n"/>
+      <c r="F132" s="9" t="n"/>
+      <c r="G132" s="9" t="n"/>
+      <c r="H132" s="10" t="inlineStr">
+        <is>
+          <t>Total semaine</t>
+        </is>
+      </c>
+      <c r="I132" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J132" s="9" t="n">
+        <v>257</v>
+      </c>
+      <c r="K132" s="9" t="n"/>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 13 — 24/08 au 30/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="26" customHeight="1">
+      <c r="A134" s="3" t="n">
         <v>46258</v>
       </c>
-      <c r="B132" s="4" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>Lundi</t>
         </is>
       </c>
-      <c r="C132" s="5" t="inlineStr">
+      <c r="C134" s="5" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
       </c>
-      <c r="D132" s="6" t="inlineStr">
+      <c r="D134" s="6" t="inlineStr">
         <is>
           <t>OFF / Repos</t>
         </is>
       </c>
-      <c r="E132" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G132" s="4" t="n">
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F134" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H132" s="7" t="inlineStr">
+      <c r="H134" s="7" t="inlineStr">
         <is>
           <t>Retour Luxembourg En Vélo — repos
 Dernier grand repos avant semaine finale</t>
         </is>
       </c>
-      <c r="I132" s="4" t="n"/>
-      <c r="J132" s="4" t="n"/>
-      <c r="K132" s="4" t="n"/>
-      <c r="L132" s="4" t="n"/>
-    </row>
-    <row r="133" ht="15" customHeight="1">
-      <c r="A133" s="9" t="n"/>
-      <c r="B133" s="9" t="n"/>
-      <c r="C133" s="9" t="n"/>
-      <c r="D133" s="9" t="n"/>
-      <c r="E133" s="9" t="n"/>
-      <c r="F133" s="9" t="n"/>
-      <c r="G133" s="9" t="n"/>
-      <c r="H133" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL PÉRIODE</t>
-        </is>
-      </c>
-      <c r="I133" s="9" t="n"/>
-      <c r="J133" s="9" t="n">
-        <v>177</v>
-      </c>
-      <c r="K133" s="9" t="n"/>
-      <c r="L133" s="9" t="n"/>
-    </row>
-    <row r="134" ht="20" customHeight="1">
-      <c r="A134" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  25/08 → 30/08/2026   |   Dernière semaine pré-plan IM | Nat WE 29-30 août</t>
-        </is>
-      </c>
+      <c r="I134" s="4" t="n"/>
+      <c r="J134" s="4" t="n"/>
+      <c r="K134" s="4" t="n"/>
     </row>
     <row r="135" ht="26" customHeight="1">
       <c r="A135" s="3" t="n">
@@ -5843,7 +5533,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C135" s="12" t="inlineStr">
+      <c r="C135" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -5875,9 +5565,6 @@
       </c>
       <c r="J135" s="4" t="n"/>
       <c r="K135" s="4" t="n"/>
-      <c r="L135" s="4" t="n">
-        <v>48</v>
-      </c>
     </row>
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="n">
@@ -5888,7 +5575,7 @@
           <t>Mardi</t>
         </is>
       </c>
-      <c r="C136" s="16" t="inlineStr">
+      <c r="C136" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5919,9 +5606,6 @@
         <v>19</v>
       </c>
       <c r="K136" s="4" t="n"/>
-      <c r="L136" s="4" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="137" ht="26" customHeight="1">
       <c r="A137" s="3" t="n">
@@ -5932,7 +5616,7 @@
           <t>Mercredi</t>
         </is>
       </c>
-      <c r="C137" s="16" t="inlineStr">
+      <c r="C137" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -5964,9 +5648,6 @@
         <v>46</v>
       </c>
       <c r="K137" s="4" t="n"/>
-      <c r="L137" s="4" t="n">
-        <v>126</v>
-      </c>
     </row>
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="n">
@@ -5977,7 +5658,7 @@
           <t>Jeudi</t>
         </is>
       </c>
-      <c r="C138" s="12" t="inlineStr">
+      <c r="C138" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -6008,9 +5689,6 @@
       </c>
       <c r="J138" s="4" t="n"/>
       <c r="K138" s="4" t="n"/>
-      <c r="L138" s="4" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="139" ht="39" customHeight="1">
       <c r="A139" s="3" t="n">
@@ -6021,7 +5699,7 @@
           <t>Vendredi</t>
         </is>
       </c>
-      <c r="C139" s="12" t="inlineStr">
+      <c r="C139" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -6054,9 +5732,6 @@
       </c>
       <c r="J139" s="4" t="n"/>
       <c r="K139" s="4" t="n"/>
-      <c r="L139" s="4" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="140" ht="26" customHeight="1">
       <c r="A140" s="3" t="n">
@@ -6067,7 +5742,7 @@
           <t>Samedi</t>
         </is>
       </c>
-      <c r="C140" s="16" t="inlineStr">
+      <c r="C140" s="12" t="inlineStr">
         <is>
           <t>Vélo</t>
         </is>
@@ -6099,9 +5774,6 @@
         <v>57</v>
       </c>
       <c r="K140" s="4" t="n"/>
-      <c r="L140" s="4" t="n">
-        <v>154</v>
-      </c>
     </row>
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="n">
@@ -6143,7 +5815,6 @@
       <c r="K141" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="L141" s="4" t="n"/>
     </row>
     <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="n">
@@ -6185,7 +5856,6 @@
       <c r="K142" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="L142" s="4" t="n"/>
     </row>
     <row r="143" ht="39" customHeight="1">
       <c r="A143" s="3" t="n">
@@ -6196,7 +5866,7 @@
           <t>Dimanche</t>
         </is>
       </c>
-      <c r="C143" s="12" t="inlineStr">
+      <c r="C143" s="11" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
@@ -6229,9 +5899,6 @@
       </c>
       <c r="J143" s="4" t="n"/>
       <c r="K143" s="4" t="n"/>
-      <c r="L143" s="4" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="144" ht="15" customHeight="1">
       <c r="A144" s="9" t="n"/>
@@ -6243,7 +5910,7 @@
       <c r="G144" s="9" t="n"/>
       <c r="H144" s="10" t="inlineStr">
         <is>
-          <t>TOTAL PÉRIODE</t>
+          <t>Total semaine</t>
         </is>
       </c>
       <c r="I144" s="9" t="n">
@@ -6255,40 +5922,22 @@
       <c r="K144" s="9" t="n">
         <v>3600</v>
       </c>
-      <c r="L144" s="9" t="n"/>
-    </row>
-    <row r="145" ht="22" customHeight="1">
-      <c r="A145" s="21" t="inlineStr">
-        <is>
-          <t>TOTAL PRÉPARATION — 3 juin → 30 août 2026</t>
-        </is>
-      </c>
-      <c r="I145" s="22" t="n">
-        <v>274</v>
-      </c>
-      <c r="J145" s="22" t="n">
-        <v>1077</v>
-      </c>
-      <c r="K145" s="22" t="n">
-        <v>25300</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A145:H145"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A82:L82"/>
-    <mergeCell ref="A134:L134"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A128:L128"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A108:L108"/>
-    <mergeCell ref="A121:L121"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A88:L88"/>
-    <mergeCell ref="A9:L9"/>
-    <mergeCell ref="A56:L56"/>
-    <mergeCell ref="A69:L69"/>
+  <mergeCells count="13">
+    <mergeCell ref="A56:K56"/>
+    <mergeCell ref="A69:K69"/>
+    <mergeCell ref="A92:K92"/>
+    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="A82:K82"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A110:K110"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A133:K133"/>
+    <mergeCell ref="A123:K123"/>
+    <mergeCell ref="A9:K9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto sync 2026-06-30 19:35:01
</commit_message>
<xml_diff>
--- a/Marathon_programme.xlsx
+++ b/Marathon_programme.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -119,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,7 +126,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -155,6 +154,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -603,7 +605,7 @@
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="13" t="n">
         <v>46176</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -647,7 +649,7 @@
       <c r="K3" s="4" t="n"/>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="13" t="n">
         <v>46177</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -689,7 +691,7 @@
       <c r="K4" s="4" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="13" t="n">
         <v>46178</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -730,7 +732,7 @@
       <c r="K5" s="4" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="13" t="n">
         <v>46179</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -774,7 +776,7 @@
       </c>
     </row>
     <row r="7" ht="39" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="13" t="n">
         <v>46180</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -843,7 +845,7 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="13" t="n">
         <v>46181</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -884,7 +886,7 @@
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11" ht="104" customHeight="1">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="13" t="n">
         <v>46182</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -932,7 +934,7 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12" ht="39" customHeight="1">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="13" t="n">
         <v>46183</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -975,7 +977,7 @@
       <c r="K12" s="4" t="n"/>
     </row>
     <row r="13" ht="91" customHeight="1">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="13" t="n">
         <v>46184</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1022,7 +1024,7 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="13" t="n">
         <v>46185</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1063,7 +1065,7 @@
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="13" t="n">
         <v>46186</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1105,7 +1107,7 @@
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="13" t="n">
         <v>46187</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1147,7 +1149,7 @@
       </c>
     </row>
     <row r="17" ht="39" customHeight="1">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="13" t="n">
         <v>46187</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1218,7 +1220,7 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="13" t="n">
         <v>46188</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1259,7 +1261,7 @@
       <c r="K20" s="4" t="n"/>
     </row>
     <row r="21" ht="65" customHeight="1">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="13" t="n">
         <v>46189</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1304,7 +1306,7 @@
       <c r="K21" s="4" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="13" t="n">
         <v>46190</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1345,7 +1347,7 @@
       <c r="K22" s="4" t="n"/>
     </row>
     <row r="23" ht="52" customHeight="1">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="13" t="n">
         <v>46191</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1389,7 +1391,7 @@
       <c r="K23" s="4" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="13" t="n">
         <v>46192</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1430,7 +1432,7 @@
       <c r="K24" s="4" t="n"/>
     </row>
     <row r="25" ht="108" customHeight="1">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="13" t="n">
         <v>46193</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1479,7 +1481,7 @@
       <c r="K25" s="4" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="13" t="n">
         <v>46194</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1547,7 +1549,7 @@
       </c>
     </row>
     <row r="29" ht="104" customHeight="1">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="13" t="n">
         <v>46195</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1595,7 +1597,7 @@
       <c r="K29" s="4" t="n"/>
     </row>
     <row r="30" ht="39" customHeight="1">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="13" t="n">
         <v>46195</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1638,7 +1640,7 @@
       </c>
     </row>
     <row r="31" ht="78" customHeight="1">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="13" t="n">
         <v>46196</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1684,7 +1686,7 @@
       <c r="K31" s="4" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="3" t="n">
+      <c r="A32" s="13" t="n">
         <v>46196</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1725,7 +1727,7 @@
       </c>
     </row>
     <row r="33" ht="78" customHeight="1">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="13" t="n">
         <v>46197</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1771,7 +1773,7 @@
       <c r="K33" s="4" t="n"/>
     </row>
     <row r="34" ht="39" customHeight="1">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="13" t="n">
         <v>46197</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1814,7 +1816,7 @@
       </c>
     </row>
     <row r="35" ht="39" customHeight="1">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="13" t="n">
         <v>46198</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1857,7 +1859,7 @@
       <c r="K35" s="4" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="3" t="n">
+      <c r="A36" s="13" t="n">
         <v>46198</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1899,7 +1901,7 @@
       </c>
     </row>
     <row r="37" ht="78" customHeight="1">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="13" t="n">
         <v>46199</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1945,7 +1947,7 @@
       <c r="K37" s="4" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="13" t="n">
         <v>46199</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1986,7 +1988,7 @@
       </c>
     </row>
     <row r="39" ht="65" customHeight="1">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="13" t="n">
         <v>46200</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2031,7 +2033,7 @@
       <c r="K39" s="4" t="n"/>
     </row>
     <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="3" t="n">
+      <c r="A40" s="13" t="n">
         <v>46200</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2073,7 +2075,7 @@
       </c>
     </row>
     <row r="41" ht="39" customHeight="1">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="13" t="n">
         <v>46201</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2144,7 +2146,7 @@
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="13" t="n">
         <v>46202</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2154,38 +2156,39 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>Repos — récup camp Malaga + voyage retour</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
+      <c r="J44" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K44" s="4" t="n"/>
     </row>
     <row r="45" ht="104" customHeight="1">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="13" t="n">
         <v>46203</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2218,11 +2221,7 @@
         <is>
           <t>RETOUR VÉLO après 7 semaines !
 55' Z2 très facile (120-133 bpm)
-PROTOCOLE GENOU :
-  · Cadence HAUTE : 90-95 rpm minimum — réduit la pression sur le genou
-  · Selle légèrement plus haute qu'habitude (1-2 cm)
-  · ZÉRO force — ZÉRO basse cadence pendant 2 semaines
-  · Plateau facile — résistance minimale
+Cadence HAUTE 90-95 rpm minimum
 Écouter les sensations du genou</t>
         </is>
       </c>
@@ -2233,7 +2232,7 @@
       <c r="K45" s="4" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="13" t="n">
         <v>46203</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2248,34 +2247,36 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>EF légère post-Malaga — plat</t>
+          <t>EF très légère test — marche-course PLAT</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>Z1-Z2</t>
+          <t>Z1</t>
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>32' EF Z2 (120-133 bpm) — terrain plat
-Post-camp Malaga — observer les sensations genou</t>
+          <t>Seule sortie course test de la semaine
+Marche-course 2min/1min, terrain plat strict, FC &lt; 128 bpm
+Si douleur bandelette/rotule &gt; 2/10 : ARRÊT
+Renfo fessier le soir obligatoire</t>
         </is>
       </c>
       <c r="I46" s="4" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="J46" s="4" t="n"/>
       <c r="K46" s="4" t="n"/>
     </row>
     <row r="47" ht="39" customHeight="1">
-      <c r="A47" s="3" t="n">
+      <c r="A47" s="13" t="n">
         <v>46204</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -2290,11 +2291,11 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 — 80' (cadence haute)</t>
+          <t>Sortie Z2 — 100' (cadence haute)</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
@@ -2306,19 +2307,19 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>80' Z2 (127-138 bpm)
-Cadence 90-95 rpm — pas de basse cadence
-NUTRITION : 40g/h si besoin</t>
+          <t>100' Z2 (127-138 bpm)
+Cadence 90-95 rpm
+NUTRITION : 42g/h</t>
         </is>
       </c>
       <c r="I47" s="4" t="n"/>
       <c r="J47" s="4" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="K47" s="4" t="n"/>
     </row>
     <row r="48" ht="52" customHeight="1">
-      <c r="A48" s="3" t="n">
+      <c r="A48" s="13" t="n">
         <v>46205</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2333,11 +2334,11 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Vélo cadence haute — 55' (pas de force)</t>
+          <t>Vélo cadence haute — 70'</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
@@ -2349,20 +2350,17 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>10' EF | 4x8' cadence HAUTE 95-100 rpm @ Z2 — r=3' | 15' RC
-PROTOCOLE GENOU : PAS de basse cadence avant 2 semaines sans douleur
-Basse cadence = forte pression genou → contre-indiqué
-Cadence haute = cardio sans pression articulaire</t>
+          <t>10' EF | 5x9' cadence HAUTE 95-100 rpm @ Z2 — r=3' | 15' RC</t>
         </is>
       </c>
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="4" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="K48" s="4" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="3" t="n">
+      <c r="A49" s="13" t="n">
         <v>46205</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -2372,38 +2370,39 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Repos</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>EF — 30' plat</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>30</v>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>Z1-Z2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile — terrain plat</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="n">
-        <v>5.5</v>
-      </c>
+          <t>Repos course — vélo le matin suffit
+Étirements + renfo fessier</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="n"/>
       <c r="J49" s="4" t="n"/>
       <c r="K49" s="4" t="n"/>
     </row>
     <row r="50" ht="26" customHeight="1">
-      <c r="A50" s="3" t="n">
+      <c r="A50" s="13" t="n">
         <v>46206</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2413,39 +2412,39 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>EF + strides — 35' plat</t>
+          <t>Vélo Z2 — 75'</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>Z1-Z2</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 | 4x20'' strides en fin
-Foncier progressif — terrain plat</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="J50" s="4" t="n"/>
+          <t>75' Z2 (127-138 bpm) — cadence 90-95 rpm
+Pas de course aujourd'hui</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="n"/>
+      <c r="J50" s="4" t="n">
+        <v>36</v>
+      </c>
       <c r="K50" s="4" t="n"/>
     </row>
     <row r="51" ht="39" customHeight="1">
-      <c r="A51" s="3" t="n">
+      <c r="A51" s="13" t="n">
         <v>46207</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -2460,11 +2459,11 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 100'</t>
+          <t>Sortie longue Z2 — 140'</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
@@ -2472,23 +2471,22 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>100' Z2 (127-138 bpm) — première vraie longue vélo
-Z2 pur — cadence 90-95 rpm — pas de blocs
-NUTRITION : 40g/h | Selle position genou OK</t>
+          <t>140' Z2 (127-138 bpm) — sortie longue compensatoire
+Cadence 90-95 rpm | NUTRITION : 48g/h</t>
         </is>
       </c>
       <c r="I51" s="4" t="n"/>
       <c r="J51" s="4" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="K51" s="4" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="3" t="n">
+      <c r="A52" s="13" t="n">
         <v>46207</v>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2529,7 +2527,7 @@
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="3" t="n">
+      <c r="A53" s="13" t="n">
         <v>46208</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -2570,7 +2568,7 @@
       </c>
     </row>
     <row r="54" ht="52" customHeight="1">
-      <c r="A54" s="3" t="n">
+      <c r="A54" s="13" t="n">
         <v>46208</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -2580,36 +2578,35 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Repos</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 62' (plat/vallonné doux)</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="n">
-        <v>62</v>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>62' Z2 (127-138 bpm) — foncier CAP
-Allure conversationnelle
-PROTOCOLE GENOU : plat ou légèrement vallonné
-Éviter les descentes raides — pentes douces uniquement</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="n">
-        <v>11.5</v>
-      </c>
+          <t>Pas de sortie longue course cette semaine
+Natation du jour suffit comme volume
+Étirements + renfo fessier</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="n"/>
       <c r="J54" s="4" t="n"/>
       <c r="K54" s="4" t="n"/>
     </row>
@@ -2644,7 +2641,7 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="3" t="n">
+      <c r="A57" s="13" t="n">
         <v>46209</v>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2654,38 +2651,39 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I57" s="4" t="n"/>
-      <c r="J57" s="4" t="n"/>
+      <c r="J57" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K57" s="4" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="3" t="n">
+      <c r="A58" s="13" t="n">
         <v>46210</v>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2700,11 +2698,11 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Vélo récup Z2 — 42'</t>
+          <t>Vélo récup Z2 — 55'</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
@@ -2716,17 +2714,17 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>42' Z2 récup — cadence souple 90-95 rpm</t>
+          <t>55' Z2 récup — cadence souple 90-95 rpm</t>
         </is>
       </c>
       <c r="I58" s="4" t="n"/>
       <c r="J58" s="4" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K58" s="4" t="n"/>
     </row>
     <row r="59" ht="52" customHeight="1">
-      <c r="A59" s="3" t="n">
+      <c r="A59" s="13" t="n">
         <v>46210</v>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2736,41 +2734,39 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Repos</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Qualité légère — Tempo 2x12'</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>50</v>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
-FC cible : 147-153 bpm — ne pas dépasser 155 bpm
-4x20'' strides en fin
-Terrain plat ou très légèrement ondulé</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="n">
-        <v>9</v>
-      </c>
+          <t>Pas de tempo — diagnostic non confirmé (rdv kiné 16/07)
+Vélo du matin suffit comme charge</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="n"/>
       <c r="J59" s="4" t="n"/>
       <c r="K59" s="4" t="n"/>
     </row>
     <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="3" t="n">
+      <c r="A60" s="13" t="n">
         <v>46211</v>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2785,11 +2781,11 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 — 90'</t>
+          <t>Sortie Z2 — 115'</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
@@ -2797,22 +2793,22 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>90' Z2 (127-138 bpm) | Cadence 88-93 rpm
-NUTRITION : 42g/h</t>
+          <t>115' Z2 (127-138 bpm) | Cadence 88-93 rpm
+NUTRITION : 44g/h</t>
         </is>
       </c>
       <c r="I60" s="4" t="n"/>
       <c r="J60" s="4" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="K60" s="4" t="n"/>
     </row>
     <row r="61" ht="78" customHeight="1">
-      <c r="A61" s="3" t="n">
+      <c r="A61" s="13" t="n">
         <v>46212</v>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2827,38 +2823,34 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Vélo cadence mixte — 65'</t>
+          <t>Vélo cadence haute — 80'</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>10' EF
-SI genou symptôme-free depuis 1 semaine :
-  4x5' basse cadence (65 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm
-SINON :
-  6x8' cadence haute 92-97 rpm @ Z2 — r=2'
-Toujours écouter le genou</t>
+          <t>10' EF | 6x9' cadence haute 92-97 rpm @ Z2 — r=2' | 10' RC
+Pas de basse cadence — genou encore sensible</t>
         </is>
       </c>
       <c r="I61" s="4" t="n"/>
       <c r="J61" s="4" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="K61" s="4" t="n"/>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="3" t="n">
+      <c r="A62" s="13" t="n">
         <v>46212</v>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -2873,33 +2865,35 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>EF — 30'</t>
+          <t>EF très léger test — 18' plat</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G62" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile — plat</t>
+          <t>Seule sortie course test de la semaine
+Terrain plat strict — si douleur &gt; 2/10 : ARRÊT
+À noter précisément pour le rdv kiné</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="J62" s="4" t="n"/>
       <c r="K62" s="4" t="n"/>
     </row>
     <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="3" t="n">
+      <c r="A63" s="13" t="n">
         <v>46213</v>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -2909,39 +2903,39 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Tempo — 2x15'</t>
+          <t>Vélo Z2 — 80'</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>12' EF | 2x15' Z3 (148-156 bpm) — r=3' | 12' RC
-FC cible : 148-156 bpm — terrain plat</t>
-        </is>
-      </c>
-      <c r="I63" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="J63" s="4" t="n"/>
+          <t>80' Z2 — cadence 90-95 rpm
+Pas de course aujourd'hui</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="n">
+        <v>39</v>
+      </c>
       <c r="K63" s="4" t="n"/>
     </row>
     <row r="64" ht="26" customHeight="1">
-      <c r="A64" s="3" t="n">
+      <c r="A64" s="13" t="n">
         <v>46214</v>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -2956,11 +2950,11 @@
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 120'</t>
+          <t>Sortie longue Z2 — 150'</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
@@ -2968,22 +2962,22 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>120' Z2 (127-140 bpm) | 2x18' Z3 inclus — r=10'
-NUTRITION : 45g/h | Cadence 88-93 rpm</t>
+          <t>150' Z2 pur (127-138 bpm)
+NUTRITION : 48g/h | Cadence 88-93 rpm</t>
         </is>
       </c>
       <c r="I64" s="4" t="n"/>
       <c r="J64" s="4" t="n">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="K64" s="4" t="n"/>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="3" t="n">
+      <c r="A65" s="13" t="n">
         <v>46214</v>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -3024,7 +3018,7 @@
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="3" t="n">
+      <c r="A66" s="13" t="n">
         <v>46215</v>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3065,7 +3059,7 @@
       </c>
     </row>
     <row r="67" ht="39" customHeight="1">
-      <c r="A67" s="3" t="n">
+      <c r="A67" s="13" t="n">
         <v>46215</v>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -3075,35 +3069,34 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Repos</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 75' (plat/vallonné doux)</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="n">
-        <v>75</v>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G67" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>75' Z2 (127-140 bpm) — foncier
-Allure conversationnelle
-Genou : éviter les descentes raides — terrain plat/légèrement vallonné</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="n">
-        <v>14</v>
-      </c>
+          <t>Pas de sortie longue course — diagnostic pas encore posé
+Natation du jour suffit comme volume</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="n"/>
       <c r="J67" s="4" t="n"/>
       <c r="K67" s="4" t="n"/>
     </row>
@@ -3138,7 +3131,7 @@
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="3" t="n">
+      <c r="A70" s="13" t="n">
         <v>46216</v>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -3148,38 +3141,39 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I70" s="4" t="n"/>
-      <c r="J70" s="4" t="n"/>
+      <c r="J70" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K70" s="4" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="3" t="n">
+      <c r="A71" s="13" t="n">
         <v>46217</v>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -3194,11 +3188,11 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Vélo récup Z2 — 42'</t>
+          <t>Vélo récup Z2 — 55'</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
@@ -3210,17 +3204,17 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>42' Z2 récup — cadence 90-95 rpm</t>
+          <t>55' Z2 récup — cadence 90-95 rpm</t>
         </is>
       </c>
       <c r="I71" s="4" t="n"/>
       <c r="J71" s="4" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K71" s="4" t="n"/>
     </row>
     <row r="72" ht="91" customHeight="1">
-      <c r="A72" s="3" t="n">
+      <c r="A72" s="13" t="n">
         <v>46217</v>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -3230,44 +3224,39 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Course</t>
+          <t>Repos</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Qualité — 4x2000m</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="n">
-        <v>60</v>
+          <t>OFF / Repos</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>Z3-Z4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>12' EF
-4x2000m progressif :
-  Rép 1-2 : 83-84% FCmax → FC 161-164 bpm
-  Rép 3-4 : 85% FCmax → FC 164-166 bpm
-r=1'30 — FC sous 145 bpm
-10' RC
-Terrain plat</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="n">
-        <v>11.5</v>
-      </c>
+          <t>RDV KINÉ DEMAIN — repos course, observer les sensations
+Noter tout pour la consultation</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="n"/>
       <c r="J72" s="4" t="n"/>
       <c r="K72" s="4" t="n"/>
     </row>
     <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="3" t="n">
+      <c r="A73" s="13" t="n">
         <v>46218</v>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -3282,15 +3271,15 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 + blocs — 105'</t>
+          <t>Sortie Z2 — 120'</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G73" s="4" t="n">
@@ -3298,18 +3287,18 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>105' Z2 | 2x18' SS @ 83% FTP — r=7'
-NUTRITION : 47g/h</t>
+          <t>120' Z2 (127-138 bpm) | Cadence 88-93 rpm
+NUTRITION : 46g/h</t>
         </is>
       </c>
       <c r="I73" s="4" t="n"/>
       <c r="J73" s="4" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="K73" s="4" t="n"/>
     </row>
     <row r="74" ht="65" customHeight="1">
-      <c r="A74" s="3" t="n">
+      <c r="A74" s="13" t="n">
         <v>46219</v>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -3324,37 +3313,35 @@
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Force vélo — 70' (si asymptomatique)</t>
+          <t>Vélo léger — 45' (jour du RDV kiné)</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G74" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>10' EF
-SI symptôme-free depuis 2 semaines → programme normal :
-  5x6' basse cadence (60 rpm) @ Z2-Z3 — r=3' + 2x5' cadence 100 rpm
-SI encore sensible → cadence haute uniquement :
-  6x8' cadence 92-97 rpm @ Z2 — r=2'</t>
+          <t>🩺 RDV KINÉ AUJOURD'HUI 16/07
+45' Z2 facile, cadence haute
+Le protocole de la suite sera ajusté selon le diagnostic</t>
         </is>
       </c>
       <c r="I74" s="4" t="n"/>
       <c r="J74" s="4" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="K74" s="4" t="n"/>
     </row>
     <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="3" t="n">
+      <c r="A75" s="13" t="n">
         <v>46219</v>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -3369,33 +3356,34 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>EF — 32'</t>
+          <t>EF — 20' (à ajuster selon avis kiné)</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>32' EF Z2 facile — plat</t>
+          <t>20' EF Z1-Z2 — terrain plat
+À AJUSTER selon diagnostic et consignes du kiné reçues le matin même</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J75" s="4" t="n"/>
       <c r="K75" s="4" t="n"/>
     </row>
     <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="3" t="n">
+      <c r="A76" s="13" t="n">
         <v>46220</v>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -3410,34 +3398,35 @@
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Tempo — 2x18'</t>
+          <t>EF — 25' (intensité selon avis kiné)</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G76" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>12' EF | 2x18' Z3 (150-158 bpm) — r=3' | 12' RC
-FC cible : 150-158 bpm — terrain plat</t>
+          <t>25' EF Z1-Z2 par défaut — terrain plat
+SI kiné valide : tempo léger 2x8' Z3 max possible
+SINON : rester en EF pur</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>10.5</v>
+        <v>4.5</v>
       </c>
       <c r="J76" s="4" t="n"/>
       <c r="K76" s="4" t="n"/>
     </row>
     <row r="77" ht="39" customHeight="1">
-      <c r="A77" s="3" t="n">
+      <c r="A77" s="13" t="n">
         <v>46221</v>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -3452,11 +3441,11 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 140' (PIC pré-vacances)</t>
+          <t>Sortie longue Z2 — 155' (PIC pré-vacances)</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
@@ -3468,19 +3457,18 @@
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>140' Z2 (127-140 bpm) — PIC avant vacances
-2x22' Z3 inclus — r=10'
-NUTRITION : 48g/h | Cadence 85-93 rpm</t>
+          <t>155' Z2 (127-140 bpm) — PIC avant vacances
+NUTRITION : 50g/h | Cadence 85-93 rpm</t>
         </is>
       </c>
       <c r="I77" s="4" t="n"/>
       <c r="J77" s="4" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="K77" s="4" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="3" t="n">
+      <c r="A78" s="13" t="n">
         <v>46221</v>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -3521,7 +3509,7 @@
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="3" t="n">
+      <c r="A79" s="13" t="n">
         <v>46222</v>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -3562,7 +3550,7 @@
       </c>
     </row>
     <row r="80" ht="39" customHeight="1">
-      <c r="A80" s="3" t="n">
+      <c r="A80" s="13" t="n">
         <v>46222</v>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -3577,11 +3565,11 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 82' (PIC pré-vacances)</t>
+          <t>Sortie longue — 35' à 55' selon avis kiné</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
@@ -3589,17 +3577,17 @@
         </is>
       </c>
       <c r="G80" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>82' Z2 (127-140 bpm) — pic avant Italie
-Allure conversationnelle
-Genou : toujours terrain plat/légèrement vallonné — descentes douces</t>
+          <t>Par défaut : 35' Z2 plat, allure conversationnelle
+SI feu vert kiné + zéro symptôme : étendre jusqu'à 55'
+Reprise progressive — pas le retour direct au volume initial (82')</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>15.5</v>
+        <v>6</v>
       </c>
       <c r="J80" s="4" t="n"/>
       <c r="K80" s="4" t="n"/>
@@ -3635,7 +3623,7 @@
       </c>
     </row>
     <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="3" t="n">
+      <c r="A83" s="13" t="n">
         <v>46223</v>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -3645,38 +3633,39 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I83" s="4" t="n"/>
-      <c r="J83" s="4" t="n"/>
+      <c r="J83" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K83" s="4" t="n"/>
     </row>
     <row r="84" ht="26" customHeight="1">
-      <c r="A84" s="3" t="n">
+      <c r="A84" s="13" t="n">
         <v>46224</v>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -3691,34 +3680,33 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>Vélo Z2 + tempo court — 60'</t>
+          <t>Vélo Z2 — 70'</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G84" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>15' EF | 20' Z3 (148-156 bpm) | 18' Z2 | 7' RC
-Dernière séance vélo avant Italie</t>
+          <t>70' Z2 — cadence haute 90-95 rpm</t>
         </is>
       </c>
       <c r="I84" s="4" t="n"/>
       <c r="J84" s="4" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="K84" s="4" t="n"/>
     </row>
     <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="3" t="n">
+      <c r="A85" s="13" t="n">
         <v>46224</v>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -3733,33 +3721,33 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>EF — 28'</t>
+          <t>EF — 22' (selon évolution post rdv kiné)</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G85" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>28' EF Z2 facile avant voyage</t>
+          <t>22' EF — réduit vs initial (28'), à ajuster selon retour kiné de la semaine précédente</t>
         </is>
       </c>
       <c r="I85" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J85" s="4" t="n"/>
       <c r="K85" s="4" t="n"/>
     </row>
     <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="3" t="n">
+      <c r="A86" s="13" t="n">
         <v>46225</v>
       </c>
       <c r="B86" s="4" t="inlineStr">
@@ -3774,11 +3762,11 @@
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 — 65'</t>
+          <t>Sortie Z2 — 80'</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
@@ -3790,17 +3778,17 @@
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>65' Z2 — courte avant voyage demain</t>
+          <t>80' Z2 — légèrement augmenté vs initial (65')</t>
         </is>
       </c>
       <c r="I86" s="4" t="n"/>
       <c r="J86" s="4" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="K86" s="4" t="n"/>
     </row>
     <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="3" t="n">
+      <c r="A87" s="13" t="n">
         <v>46226</v>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -3841,7 +3829,7 @@
       <c r="K87" s="4" t="n"/>
     </row>
     <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="3" t="n">
+      <c r="A88" s="13" t="n">
         <v>46227</v>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -3882,7 +3870,7 @@
       <c r="K88" s="4" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="3" t="n">
+      <c r="A89" s="13" t="n">
         <v>46228</v>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -3923,7 +3911,7 @@
       <c r="K89" s="4" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="3" t="n">
+      <c r="A90" s="13" t="n">
         <v>46229</v>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -3992,7 +3980,7 @@
       </c>
     </row>
     <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="3" t="n">
+      <c r="A93" s="13" t="n">
         <v>46230</v>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -4025,7 +4013,7 @@
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>🇮🇹 Rome — ZÉRO SÉANCE</t>
+          <t>Vacances Italie/Grèce</t>
         </is>
       </c>
       <c r="I93" s="4" t="n"/>
@@ -4033,7 +4021,7 @@
       <c r="K93" s="4" t="n"/>
     </row>
     <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="3" t="n">
+      <c r="A94" s="13" t="n">
         <v>46231</v>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -4074,7 +4062,7 @@
       <c r="K94" s="4" t="n"/>
     </row>
     <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="3" t="n">
+      <c r="A95" s="13" t="n">
         <v>46232</v>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -4115,7 +4103,7 @@
       <c r="K95" s="4" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="3" t="n">
+      <c r="A96" s="13" t="n">
         <v>46233</v>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -4156,7 +4144,7 @@
       <c r="K96" s="4" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="3" t="n">
+      <c r="A97" s="13" t="n">
         <v>46234</v>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -4197,7 +4185,7 @@
       <c r="K97" s="4" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="3" t="n">
+      <c r="A98" s="13" t="n">
         <v>46235</v>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -4238,7 +4226,7 @@
       <c r="K98" s="4" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
-      <c r="A99" s="3" t="n">
+      <c r="A99" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -4303,7 +4291,7 @@
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="3" t="n">
+      <c r="A102" s="13" t="n">
         <v>46237</v>
       </c>
       <c r="B102" s="4" t="inlineStr">
@@ -4336,7 +4324,7 @@
       </c>
       <c r="H102" s="7" t="inlineStr">
         <is>
-          <t>🇬🇷 Grèce avec maman — ZÉRO SÉANCE</t>
+          <t>Vacances Italie/Grèce</t>
         </is>
       </c>
       <c r="I102" s="4" t="n"/>
@@ -4344,7 +4332,7 @@
       <c r="K102" s="4" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="3" t="n">
+      <c r="A103" s="13" t="n">
         <v>46238</v>
       </c>
       <c r="B103" s="4" t="inlineStr">
@@ -4385,7 +4373,7 @@
       <c r="K103" s="4" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="3" t="n">
+      <c r="A104" s="13" t="n">
         <v>46239</v>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -4426,7 +4414,7 @@
       <c r="K104" s="4" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="3" t="n">
+      <c r="A105" s="13" t="n">
         <v>46240</v>
       </c>
       <c r="B105" s="4" t="inlineStr">
@@ -4467,7 +4455,7 @@
       <c r="K105" s="4" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
-      <c r="A106" s="3" t="n">
+      <c r="A106" s="13" t="n">
         <v>46241</v>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -4508,7 +4496,7 @@
       <c r="K106" s="4" t="n"/>
     </row>
     <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="3" t="n">
+      <c r="A107" s="13" t="n">
         <v>46242</v>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -4549,7 +4537,7 @@
       <c r="K107" s="4" t="n"/>
     </row>
     <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="3" t="n">
+      <c r="A108" s="13" t="n">
         <v>46243</v>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -4614,7 +4602,7 @@
       </c>
     </row>
     <row r="111" ht="91" customHeight="1">
-      <c r="A111" s="3" t="n">
+      <c r="A111" s="13" t="n">
         <v>46244</v>
       </c>
       <c r="B111" s="4" t="inlineStr">
@@ -4624,87 +4612,81 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E111" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F111" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G111" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H111" s="7" t="inlineStr">
+        <is>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="n"/>
+      <c r="J111" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K111" s="4" t="n"/>
+    </row>
+    <row r="112" ht="52" customHeight="1">
+      <c r="A112" s="13" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>EF reprise — 25' plat (post-vacances)</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>Z1-Z2</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H111" s="7" t="inlineStr">
-        <is>
-          <t>Repos — récup voyage retour Grèce
-J-21 plan Ironman — reprise ultra-progressive
-STRATÉGIE 3 SEMAINES :
-Sem 1 (10-16) : RPE max 5/10 — reconstruire les automatismes
-Sem 2 (17-23) : Luxembourg vélo → boost cardiovasculaire clé
-Sem 3 (24-30) : Volume -20% — arriver FRAIS le 31 août</t>
-        </is>
-      </c>
-      <c r="I111" s="4" t="n"/>
-      <c r="J111" s="4" t="n"/>
-      <c r="K111" s="4" t="n"/>
-    </row>
-    <row r="112" ht="52" customHeight="1">
-      <c r="A112" s="3" t="n">
-        <v>46245</v>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>Mardi</t>
-        </is>
-      </c>
-      <c r="C112" s="11" t="inlineStr">
-        <is>
-          <t>Course</t>
-        </is>
-      </c>
-      <c r="D112" s="6" t="inlineStr">
-        <is>
-          <t>EF reprise — post-vacances plat</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="F112" s="6" t="inlineStr">
-        <is>
-          <t>Z1-Z2</t>
-        </is>
-      </c>
-      <c r="G112" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>35' EF Z2 (120-133 bpm) — reprise très douce
-18 jours sans séance — ne pas forcer
-Terrain plat — surveiller le genou
-Marche-course si besoin</t>
+          <t>Reprise douce après vacances — terrain plat strict
+Volume réduit vs programme initial (35')</t>
         </is>
       </c>
       <c r="I112" s="4" t="n">
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="J112" s="4" t="n"/>
       <c r="K112" s="4" t="n"/>
     </row>
     <row r="113" ht="39" customHeight="1">
-      <c r="A113" s="3" t="n">
+      <c r="A113" s="13" t="n">
         <v>46245</v>
       </c>
       <c r="B113" s="4" t="inlineStr">
@@ -4719,11 +4701,11 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>Vélo reprise Z2 — 48' (cadence haute)</t>
+          <t>Vélo reprise Z2 — 60' (cadence haute)</t>
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
@@ -4735,19 +4717,17 @@
       </c>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>48' Z2 — reprendre les jambes vélo
-Cadence 90-95 rpm — jamais &gt; Z2
-Genou : cadence haute encore obligatoire</t>
+          <t>60' Z2 — cadence haute 90-95 rpm</t>
         </is>
       </c>
       <c r="I113" s="4" t="n"/>
       <c r="J113" s="4" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="K113" s="4" t="n"/>
     </row>
     <row r="114" ht="39" customHeight="1">
-      <c r="A114" s="3" t="n">
+      <c r="A114" s="13" t="n">
         <v>46246</v>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -4762,15 +4742,15 @@
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>Sortie Z2 + SS reprise — 115'</t>
+          <t>Sortie Z2 + SS reprise — 130'</t>
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G114" s="4" t="n">
@@ -4778,19 +4758,18 @@
       </c>
       <c r="H114" s="7" t="inlineStr">
         <is>
-          <t>20' EF | 2x20' SS @ 81% FTP — r=6' | Z2 reste | 15' RC
-Reprise progressive — intensité réduite
-NUTRITION : 43g/h</t>
+          <t>130' Z2 avec quelques blocs Sweet Spot courts si asymptomatique
+Cadence 88-93 rpm</t>
         </is>
       </c>
       <c r="I114" s="4" t="n"/>
       <c r="J114" s="4" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="K114" s="4" t="n"/>
     </row>
     <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="3" t="n">
+      <c r="A115" s="13" t="n">
         <v>46247</v>
       </c>
       <c r="B115" s="4" t="inlineStr">
@@ -4805,15 +4784,15 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>EF — 33' plat</t>
+          <t>EF — 28' plat</t>
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G115" s="4" t="n">
@@ -4821,17 +4800,17 @@
       </c>
       <c r="H115" s="7" t="inlineStr">
         <is>
-          <t>33' EF Z2 facile — terrain plat</t>
+          <t>28' EF plat — légèrement sous le volume initial (33')</t>
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J115" s="4" t="n"/>
       <c r="K115" s="4" t="n"/>
     </row>
     <row r="116" ht="52" customHeight="1">
-      <c r="A116" s="3" t="n">
+      <c r="A116" s="13" t="n">
         <v>46248</v>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -4846,15 +4825,15 @@
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>Force légère — 60' (si asymptomatique)</t>
+          <t>Force légère — 75' (si asymptomatique)</t>
         </is>
       </c>
       <c r="E116" s="4" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F116" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G116" s="4" t="n">
@@ -4862,20 +4841,17 @@
       </c>
       <c r="H116" s="7" t="inlineStr">
         <is>
-          <t>10' EF
-SI genou asymptomatique :
-  4x6' basse cadence (60 rpm) @ Z2 — r=3' + 2x5' cadence 100 rpm
-SINON : cadence haute 92-97 rpm uniquement</t>
+          <t>75' Z2 — force légère cadence modérée si genou stable</t>
         </is>
       </c>
       <c r="I116" s="4" t="n"/>
       <c r="J116" s="4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="K116" s="4" t="n"/>
     </row>
     <row r="117" ht="39" customHeight="1">
-      <c r="A117" s="3" t="n">
+      <c r="A117" s="13" t="n">
         <v>46248</v>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -4890,35 +4866,35 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>Tempo très léger — 2x12'</t>
+          <t>EF — 25' (tempo très léger si feu vert)</t>
         </is>
       </c>
       <c r="E117" s="4" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="F117" s="6" t="inlineStr">
         <is>
-          <t>Z3</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H117" s="7" t="inlineStr">
         <is>
-          <t>12' EF | 2x12' Z3 (147-153 bpm) — r=3' | 12' RC
-Post-vacances — très contrôlé
-FC cible : 147-153 bpm max — terrain plat</t>
+          <t>25' EF par défaut
+Si totalement asymptomatique depuis 2 semaines : 2x8' Z3 max possible
+Sinon rester en EF pur — pas de retour direct au tempo plein (2x12')</t>
         </is>
       </c>
       <c r="I117" s="4" t="n">
-        <v>8.5</v>
+        <v>4.5</v>
       </c>
       <c r="J117" s="4" t="n"/>
       <c r="K117" s="4" t="n"/>
     </row>
     <row r="118" ht="26" customHeight="1">
-      <c r="A118" s="3" t="n">
+      <c r="A118" s="13" t="n">
         <v>46249</v>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -4933,11 +4909,11 @@
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 140'</t>
+          <t>Sortie longue Z2 — 155'</t>
         </is>
       </c>
       <c r="E118" s="4" t="n">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="F118" s="6" t="inlineStr">
         <is>
@@ -4949,18 +4925,18 @@
       </c>
       <c r="H118" s="7" t="inlineStr">
         <is>
-          <t>140' Z2 (127-140 bpm) | 2x22' Z3 inclus — r=10'
-NUTRITION : 47g/h | Cadence 85-92 rpm</t>
+          <t>155' Z2 — sortie longue compensatoire renforcée
+NUTRITION : 50g/h</t>
         </is>
       </c>
       <c r="I118" s="4" t="n"/>
       <c r="J118" s="4" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="K118" s="4" t="n"/>
     </row>
     <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="3" t="n">
+      <c r="A119" s="13" t="n">
         <v>46249</v>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -5001,7 +4977,7 @@
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="3" t="n">
+      <c r="A120" s="13" t="n">
         <v>46250</v>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -5042,7 +5018,7 @@
       </c>
     </row>
     <row r="121" ht="39" customHeight="1">
-      <c r="A121" s="3" t="n">
+      <c r="A121" s="13" t="n">
         <v>46250</v>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -5057,11 +5033,11 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>Sortie longue Z2 — 78' (plat/vallonné)</t>
+          <t>Sortie longue Z2 — 50' (plat/vallonné doux)</t>
         </is>
       </c>
       <c r="E121" s="4" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="F121" s="6" t="inlineStr">
         <is>
@@ -5069,17 +5045,16 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>78' Z2 (127-140 bpm) — foncier solide
-Allure conversationnelle
-Genou : terrain plat ou légèrement vallonné</t>
+          <t>50' Z2 — reprise progressive, bien en dessous du volume initial (78')
+Descentes douces uniquement</t>
         </is>
       </c>
       <c r="I121" s="4" t="n">
-        <v>14.5</v>
+        <v>9</v>
       </c>
       <c r="J121" s="4" t="n"/>
       <c r="K121" s="4" t="n"/>
@@ -5115,7 +5090,7 @@
       </c>
     </row>
     <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="3" t="n">
+      <c r="A124" s="13" t="n">
         <v>46251</v>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -5125,38 +5100,39 @@
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F124" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H124" s="7" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I124" s="4" t="n"/>
-      <c r="J124" s="4" t="n"/>
+      <c r="J124" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K124" s="4" t="n"/>
     </row>
     <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="3" t="n">
+      <c r="A125" s="13" t="n">
         <v>46252</v>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -5197,7 +5173,7 @@
       <c r="K125" s="4" t="n"/>
     </row>
     <row r="126" ht="91" customHeight="1">
-      <c r="A126" s="3" t="n">
+      <c r="A126" s="13" t="n">
         <v>46252</v>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -5212,39 +5188,34 @@
       </c>
       <c r="D126" s="6" t="inlineStr">
         <is>
-          <t>Qualité — 5x2000m progressif</t>
+          <t>Qualité légère — 3x1500m progressif</t>
         </is>
       </c>
       <c r="E126" s="4" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="F126" s="6" t="inlineStr">
         <is>
-          <t>Z3-Z4</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H126" s="7" t="inlineStr">
         <is>
-          <t>12' EF
-5x2000m progressif :
-  Rép 1 : 81% → FC 158-160 bpm
-  Rép 2-3 : 83% → FC 161-164 bpm
-  Rép 4-5 : 85% → FC 164-166 bpm
-r=1'30 — FC sous 145 bpm
-10' RC — terrain plat</t>
+          <t>Reprise très progressive de l'intensité — volume réduit vs initial (5x2000m)
+À faire seulement si 2 semaines sans symptôme</t>
         </is>
       </c>
       <c r="I126" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J126" s="4" t="n"/>
       <c r="K126" s="4" t="n"/>
     </row>
     <row r="127" ht="26" customHeight="1">
-      <c r="A127" s="3" t="n">
+      <c r="A127" s="13" t="n">
         <v>46253</v>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -5286,7 +5257,7 @@
       <c r="K127" s="4" t="n"/>
     </row>
     <row r="128" ht="18" customHeight="1">
-      <c r="A128" s="3" t="n">
+      <c r="A128" s="13" t="n">
         <v>46254</v>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -5301,15 +5272,15 @@
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>EF — 30'</t>
+          <t>EF — 28'</t>
         </is>
       </c>
       <c r="E128" s="4" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F128" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
@@ -5317,17 +5288,17 @@
       </c>
       <c r="H128" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 — économiser pour Luxembourg vélo</t>
+          <t>28' EF — légèrement réduit vs initial (30')</t>
         </is>
       </c>
       <c r="I128" s="4" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="J128" s="4" t="n"/>
       <c r="K128" s="4" t="n"/>
     </row>
     <row r="129" ht="39" customHeight="1">
-      <c r="A129" s="3" t="n">
+      <c r="A129" s="13" t="n">
         <v>46255</v>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -5370,7 +5341,7 @@
       <c r="K129" s="4" t="n"/>
     </row>
     <row r="130" ht="39" customHeight="1">
-      <c r="A130" s="3" t="n">
+      <c r="A130" s="13" t="n">
         <v>46256</v>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -5413,7 +5384,7 @@
       <c r="K130" s="4" t="n"/>
     </row>
     <row r="131" ht="26" customHeight="1">
-      <c r="A131" s="3" t="n">
+      <c r="A131" s="13" t="n">
         <v>46257</v>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -5483,7 +5454,7 @@
       </c>
     </row>
     <row r="134" ht="26" customHeight="1">
-      <c r="A134" s="3" t="n">
+      <c r="A134" s="13" t="n">
         <v>46258</v>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -5493,39 +5464,39 @@
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Repos</t>
+          <t>Vélo</t>
         </is>
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>OFF / Repos</t>
-        </is>
-      </c>
-      <c r="E134" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Trajet vélo boulot — 20km</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="F134" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Z2</t>
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>Retour Luxembourg En Vélo — repos
-Dernier grand repos avant semaine finale</t>
+          <t>20km trajet domicile-travail — cadence haute, allure tranquille
+Cadence 90-95 rpm — zéro force</t>
         </is>
       </c>
       <c r="I134" s="4" t="n"/>
-      <c r="J134" s="4" t="n"/>
+      <c r="J134" s="4" t="n">
+        <v>20</v>
+      </c>
       <c r="K134" s="4" t="n"/>
     </row>
     <row r="135" ht="26" customHeight="1">
-      <c r="A135" s="3" t="n">
+      <c r="A135" s="13" t="n">
         <v>46259</v>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -5540,34 +5511,34 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>Activation qualité courte</t>
+          <t>Activation qualité courte — réduite</t>
         </is>
       </c>
       <c r="E135" s="4" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="F135" s="6" t="inlineStr">
         <is>
-          <t>Z2-Z3</t>
+          <t>Z3</t>
         </is>
       </c>
       <c r="G135" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>12' EF | 15' Z3 (148-154 bpm) | 15' Z2 | 6' RC
-Activation fraîche post-Luxembourg — terrain plat</t>
+          <t>Activation légère réduite vs initial (48')
+À ajuster selon les 6 semaines précédentes</t>
         </is>
       </c>
       <c r="I135" s="4" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="J135" s="4" t="n"/>
       <c r="K135" s="4" t="n"/>
     </row>
     <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="3" t="n">
+      <c r="A136" s="13" t="n">
         <v>46259</v>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -5608,7 +5579,7 @@
       <c r="K136" s="4" t="n"/>
     </row>
     <row r="137" ht="26" customHeight="1">
-      <c r="A137" s="3" t="n">
+      <c r="A137" s="13" t="n">
         <v>46260</v>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -5650,7 +5621,7 @@
       <c r="K137" s="4" t="n"/>
     </row>
     <row r="138" ht="18" customHeight="1">
-      <c r="A138" s="3" t="n">
+      <c r="A138" s="13" t="n">
         <v>46261</v>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -5665,15 +5636,15 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>EF — 30' plat</t>
+          <t>EF — 28' plat</t>
         </is>
       </c>
       <c r="E138" s="4" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F138" s="6" t="inlineStr">
         <is>
-          <t>Z2</t>
+          <t>Z1-Z2</t>
         </is>
       </c>
       <c r="G138" s="4" t="n">
@@ -5681,17 +5652,17 @@
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 facile — terrain plat</t>
+          <t>28' EF — légèrement réduit</t>
         </is>
       </c>
       <c r="I138" s="4" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="J138" s="4" t="n"/>
       <c r="K138" s="4" t="n"/>
     </row>
     <row r="139" ht="39" customHeight="1">
-      <c r="A139" s="3" t="n">
+      <c r="A139" s="13" t="n">
         <v>46262</v>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -5706,11 +5677,11 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>EF + strides — activation finale</t>
+          <t>EF + strides légers — activation finale</t>
         </is>
       </c>
       <c r="E139" s="4" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F139" s="6" t="inlineStr">
         <is>
@@ -5722,19 +5693,18 @@
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>30' EF Z2 | 4x20'' strides (r=40'')
-Dernière sortie CAP avant le plan IM
-Lundi 31 août : l'aventure Ironman commence 💪</t>
+          <t>32' EF avec strides courts si totalement asymptomatique
+Sinon EF pur sans strides</t>
         </is>
       </c>
       <c r="I139" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J139" s="4" t="n"/>
       <c r="K139" s="4" t="n"/>
     </row>
     <row r="140" ht="26" customHeight="1">
-      <c r="A140" s="3" t="n">
+      <c r="A140" s="13" t="n">
         <v>46263</v>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -5776,7 +5746,7 @@
       <c r="K140" s="4" t="n"/>
     </row>
     <row r="141" ht="18" customHeight="1">
-      <c r="A141" s="3" t="n">
+      <c r="A141" s="13" t="n">
         <v>46263</v>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -5817,7 +5787,7 @@
       </c>
     </row>
     <row r="142" ht="18" customHeight="1">
-      <c r="A142" s="3" t="n">
+      <c r="A142" s="13" t="n">
         <v>46264</v>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -5858,7 +5828,7 @@
       </c>
     </row>
     <row r="143" ht="39" customHeight="1">
-      <c r="A143" s="3" t="n">
+      <c r="A143" s="13" t="n">
         <v>46264</v>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -5873,11 +5843,11 @@
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>🏁 Dernière sortie pré-plan IM — 72'</t>
+          <t>🏁 Dernière sortie pré-plan IM — 60'</t>
         </is>
       </c>
       <c r="E143" s="4" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="F143" s="6" t="inlineStr">
         <is>
@@ -5885,17 +5855,16 @@
         </is>
       </c>
       <c r="G143" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>72' Z2 (127-138 bpm) — dernière longue CAP
-Demain lundi 31 août : Semaine 1 du plan Ironman
-Tu as construit le socle malgré les galères — bravo 💪</t>
+          <t>60' Z2 — réduit vs initial (72') par prudence
+Dernière sortie avant le début du plan Ironman le 31/08</t>
         </is>
       </c>
       <c r="I143" s="4" t="n">
-        <v>13.5</v>
+        <v>11</v>
       </c>
       <c r="J143" s="4" t="n"/>
       <c r="K143" s="4" t="n"/>
@@ -5925,8 +5894,8 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A69:K69"/>
     <mergeCell ref="A56:K56"/>
-    <mergeCell ref="A69:K69"/>
     <mergeCell ref="A92:K92"/>
     <mergeCell ref="A101:K101"/>
     <mergeCell ref="A82:K82"/>

</xml_diff>